<commit_message>
Reestiliza card do camp e adiciona aula da planilha
</commit_message>
<xml_diff>
--- a/assets/downloads/CONTROLE DE LINES PARA COACH E ANALISTA .xlsx
+++ b/assets/downloads/CONTROLE DE LINES PARA COACH E ANALISTA .xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/649e81239f5e0a86/Imagens/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fall_\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7292EE64-F9E9-42D3-8A15-B2DB63BA6577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2721CF46-75C1-46C4-B220-C6AC57185867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{9C6B5532-5592-4A9E-A144-3055C384FDE2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{9C6B5532-5592-4A9E-A144-3055C384FDE2}"/>
   </bookViews>
   <sheets>
     <sheet name="DADOS DO TIME" sheetId="1" r:id="rId1"/>
     <sheet name="RESULTADO" sheetId="2" r:id="rId2"/>
-    <sheet name="RESULTADO DE TODOS  OS TREINOS" sheetId="3" r:id="rId3"/>
+    <sheet name="RESULTADO DE TODOS OS TREINOS" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="60">
   <si>
     <t>POSIÇÃO E ABATES</t>
   </si>
@@ -68,9 +68,6 @@
   </si>
   <si>
     <t>JOGADORES</t>
-  </si>
-  <si>
-    <t>ABATES</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -215,9 +212,6 @@
   </si>
   <si>
     <t>RESERVA 1</t>
-  </si>
-  <si>
-    <t>RESERVA 2</t>
   </si>
   <si>
     <t>RESERVA 3</t>
@@ -1049,6 +1043,178 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0" hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="21" fontId="2" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="21" fontId="2" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="21" fontId="2" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="21" fontId="2" fillId="5" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="5" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="10" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="1"/>
@@ -1057,6 +1223,74 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
@@ -1064,246 +1298,6 @@
     <xf numFmtId="2" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="21" fontId="2" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="21" fontId="2" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="21" fontId="2" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="21" fontId="2" fillId="5" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="5" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="10" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1538,9 +1532,6 @@
                 <c:pt idx="4">
                   <c:v>RESERVA 1</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>RESERVA 2</c:v>
-                </c:pt>
                 <c:pt idx="6">
                   <c:v>RESERVA 3</c:v>
                 </c:pt>
@@ -1628,9 +1619,6 @@
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>RESERVA 1</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>RESERVA 2</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>RESERVA 3</c:v>
@@ -1722,9 +1710,6 @@
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>RESERVA 1</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>RESERVA 2</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>RESERVA 3</c:v>
@@ -1837,9 +1822,6 @@
                 <c:pt idx="4">
                   <c:v>RESERVA 1</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>RESERVA 2</c:v>
-                </c:pt>
                 <c:pt idx="6">
                   <c:v>RESERVA 3</c:v>
                 </c:pt>
@@ -1951,9 +1933,6 @@
                 <c:pt idx="4">
                   <c:v>RESERVA 1</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>RESERVA 2</c:v>
-                </c:pt>
                 <c:pt idx="6">
                   <c:v>RESERVA 3</c:v>
                 </c:pt>
@@ -2042,9 +2021,6 @@
                 <c:pt idx="4">
                   <c:v>RESERVA 1</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>RESERVA 2</c:v>
-                </c:pt>
                 <c:pt idx="6">
                   <c:v>RESERVA 3</c:v>
                 </c:pt>
@@ -2133,9 +2109,6 @@
                 <c:pt idx="4">
                   <c:v>RESERVA 1</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>RESERVA 2</c:v>
-                </c:pt>
                 <c:pt idx="6">
                   <c:v>RESERVA 3</c:v>
                 </c:pt>
@@ -2224,9 +2197,6 @@
                 <c:pt idx="4">
                   <c:v>RESERVA 1</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>RESERVA 2</c:v>
-                </c:pt>
                 <c:pt idx="6">
                   <c:v>RESERVA 3</c:v>
                 </c:pt>
@@ -2315,9 +2285,6 @@
                 <c:pt idx="4">
                   <c:v>RESERVA 1</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>RESERVA 2</c:v>
-                </c:pt>
                 <c:pt idx="6">
                   <c:v>RESERVA 3</c:v>
                 </c:pt>
@@ -2406,9 +2373,6 @@
                 <c:pt idx="4">
                   <c:v>RESERVA 1</c:v>
                 </c:pt>
-                <c:pt idx="5">
-                  <c:v>RESERVA 2</c:v>
-                </c:pt>
                 <c:pt idx="6">
                   <c:v>RESERVA 3</c:v>
                 </c:pt>
@@ -2431,6 +2395,9 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
+                <c:pt idx="5">
+                  <c:v>2</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -2944,11 +2911,21 @@
             <c:idx val="10"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000008-03C8-466A-929B-92A7C2E8C083}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="11"/>
             <c:invertIfNegative val="0"/>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-03C8-466A-929B-92A7C2E8C083}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
             <c:spPr>
@@ -3025,7 +3002,7 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>'RESULTADO DE TODOS  OS TREINOS'!$C$5:$C$16</c:f>
+              <c:f>'RESULTADO DE TODOS OS TREINOS'!$C$5:$C$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
@@ -3034,7 +3011,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'RESULTADO DE TODOS  OS TREINOS'!$E$5:$E$16</c:f>
+              <c:f>'RESULTADO DE TODOS OS TREINOS'!$E$5:$E$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
@@ -3128,7 +3105,7 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>'RESULTADO DE TODOS  OS TREINOS'!$C$5:$C$16</c:f>
+              <c:f>'RESULTADO DE TODOS OS TREINOS'!$C$5:$C$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
@@ -3137,7 +3114,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'RESULTADO DE TODOS  OS TREINOS'!$F$5:$F$16</c:f>
+              <c:f>'RESULTADO DE TODOS OS TREINOS'!$F$5:$F$16</c:f>
               <c:numCache>
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="12"/>
@@ -4461,15 +4438,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>734785</xdr:colOff>
+      <xdr:colOff>776076</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>176893</xdr:rowOff>
+      <xdr:rowOff>163285</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>707572</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>54429</xdr:rowOff>
+      <xdr:colOff>734787</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>217715</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4499,8 +4476,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="23309035" y="176893"/>
-          <a:ext cx="1905001" cy="2068286"/>
+          <a:off x="23350326" y="163285"/>
+          <a:ext cx="1890925" cy="1905001"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4695,7 +4672,7 @@
               <a:cs typeface="Segoe UI Semibold" panose="020B0702040204020203" pitchFamily="34" charset="0"/>
             </a:rPr>
             <a:pPr algn="ctr"/>
-            <a:t>DE 0 PARTIDAS JOGADAS O TIME ACUMULOU UM TOTAL DE 0 KILLS, E FICOU ENTRE OS 3 PRIMEIROS  0 VEZ(ES)!</a:t>
+            <a:t>DE 1 PARTIDAS JOGADAS O TIME ACUMULOU UM TOTAL DE 2 KILLS, E FICOU ENTRE OS 3 PRIMEIROS  1 VEZ(ES)!</a:t>
           </a:fld>
           <a:endParaRPr lang="en-US" sz="2400" b="1" i="1">
             <a:solidFill>
@@ -5351,7 +5328,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B7CC1EB-2F69-4734-B842-793C5114674B}">
-  <dimension ref="B1:Z49"/>
+  <dimension ref="A1:Z49"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" style="1" customWidth="1"/>
@@ -5365,9 +5342,9 @@
     <col min="21" max="21" width="12.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="29" style="1" customWidth="1"/>
     <col min="23" max="23" width="13.140625" style="1" customWidth="1"/>
-    <col min="24" max="24" width="9.85546875" style="1" hidden="1"/>
-    <col min="25" max="25" width="12.42578125" style="1" hidden="1"/>
-    <col min="26" max="26" width="7.42578125" style="1" hidden="1"/>
+    <col min="24" max="24" width="9.85546875" style="1" hidden="1" customWidth="1"/>
+    <col min="25" max="25" width="12.42578125" style="1" hidden="1" customWidth="1"/>
+    <col min="26" max="26" width="7.42578125" style="1" hidden="1" customWidth="1"/>
     <col min="27" max="16384" width="9.140625" style="1" hidden="1"/>
   </cols>
   <sheetData>
@@ -5391,352 +5368,388 @@
     </row>
     <row r="3" spans="2:20" ht="26.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="2"/>
-      <c r="C3" s="92" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3" s="93"/>
-      <c r="E3" s="93"/>
-      <c r="F3" s="93"/>
-      <c r="G3" s="93"/>
-      <c r="H3" s="93"/>
-      <c r="I3" s="93"/>
-      <c r="J3" s="93"/>
-      <c r="K3" s="93"/>
-      <c r="L3" s="93"/>
-      <c r="M3" s="93"/>
-      <c r="N3" s="93"/>
-      <c r="O3" s="94"/>
+      <c r="C3" s="76" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="77"/>
+      <c r="E3" s="77"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
+      <c r="I3" s="77"/>
+      <c r="J3" s="77"/>
+      <c r="K3" s="77"/>
+      <c r="L3" s="77"/>
+      <c r="M3" s="77"/>
+      <c r="N3" s="77"/>
+      <c r="O3" s="78"/>
       <c r="P3" s="2"/>
-      <c r="S3" s="44" t="s">
+      <c r="S3" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="T3" s="45" t="s">
+      <c r="T3" s="36" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="2:20" ht="26.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="2"/>
-      <c r="C4" s="40" t="s">
+      <c r="C4" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="41" t="s">
+      <c r="D4" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="41" t="s">
+      <c r="E4" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="41" t="s">
+      <c r="F4" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="41" t="s">
+      <c r="G4" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="41" t="s">
+      <c r="H4" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="41" t="s">
-        <v>53</v>
-      </c>
-      <c r="J4" s="41" t="s">
+      <c r="I4" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="J4" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="41" t="s">
+      <c r="K4" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="L4" s="41" t="s">
+      <c r="L4" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="M4" s="41" t="s">
+      <c r="M4" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="N4" s="41" t="s">
+      <c r="N4" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="O4" s="41" t="s">
-        <v>53</v>
+      <c r="O4" s="32" t="s">
+        <v>52</v>
       </c>
       <c r="P4" s="2"/>
-      <c r="S4" s="47">
+      <c r="S4" s="38">
         <v>1</v>
       </c>
-      <c r="T4" s="46">
+      <c r="T4" s="37">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="2:20" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="2"/>
-      <c r="C5" s="40" t="s">
+      <c r="C5" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="41"/>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="41"/>
-      <c r="I5" s="41"/>
-      <c r="J5" s="41"/>
-      <c r="K5" s="41"/>
-      <c r="L5" s="41"/>
-      <c r="M5" s="41"/>
-      <c r="N5" s="41"/>
-      <c r="O5" s="41"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+      <c r="L5" s="32"/>
+      <c r="M5" s="32"/>
+      <c r="N5" s="32"/>
+      <c r="O5" s="32">
+        <v>3</v>
+      </c>
       <c r="P5" s="2"/>
-      <c r="S5" s="47">
+      <c r="S5" s="38">
         <v>2</v>
       </c>
-      <c r="T5" s="46">
+      <c r="T5" s="37">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="2:20" ht="26.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="2"/>
-      <c r="C6" s="40" t="s">
+      <c r="C6" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="39" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="39"/>
-      <c r="F6" s="39"/>
-      <c r="G6" s="39"/>
-      <c r="H6" s="39"/>
-      <c r="I6" s="39"/>
-      <c r="J6" s="39"/>
-      <c r="K6" s="39"/>
-      <c r="L6" s="39"/>
-      <c r="M6" s="39"/>
-      <c r="N6" s="39"/>
-      <c r="O6" s="39"/>
+      <c r="D6" s="79"/>
+      <c r="E6" s="79"/>
+      <c r="F6" s="79"/>
+      <c r="G6" s="79"/>
+      <c r="H6" s="79"/>
+      <c r="I6" s="79"/>
+      <c r="J6" s="79"/>
+      <c r="K6" s="79"/>
+      <c r="L6" s="79"/>
+      <c r="M6" s="79"/>
+      <c r="N6" s="79"/>
+      <c r="O6" s="79"/>
       <c r="P6" s="2"/>
-      <c r="S6" s="47">
+      <c r="S6" s="38">
         <v>3</v>
       </c>
-      <c r="T6" s="46">
+      <c r="T6" s="37">
         <v>8</v>
       </c>
     </row>
     <row r="7" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2"/>
-      <c r="C7" s="41" t="s">
-        <v>54</v>
-      </c>
-      <c r="D7" s="41"/>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="41"/>
-      <c r="I7" s="41"/>
-      <c r="J7" s="41"/>
-      <c r="K7" s="41"/>
-      <c r="L7" s="41"/>
-      <c r="M7" s="41"/>
-      <c r="N7" s="41"/>
-      <c r="O7" s="41"/>
+      <c r="C7" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
+      <c r="J7" s="32"/>
+      <c r="K7" s="32"/>
+      <c r="L7" s="32"/>
+      <c r="M7" s="32"/>
+      <c r="N7" s="32"/>
+      <c r="O7" s="32"/>
       <c r="P7" s="2"/>
-      <c r="S7" s="47">
+      <c r="S7" s="38">
         <v>4</v>
       </c>
-      <c r="T7" s="46">
+      <c r="T7" s="37">
         <v>7</v>
       </c>
     </row>
     <row r="8" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="2"/>
-      <c r="C8" s="41" t="s">
-        <v>55</v>
-      </c>
-      <c r="D8" s="41"/>
-      <c r="E8" s="41"/>
-      <c r="F8" s="41"/>
-      <c r="G8" s="41"/>
-      <c r="H8" s="41"/>
-      <c r="I8" s="41"/>
-      <c r="J8" s="41"/>
-      <c r="K8" s="41"/>
-      <c r="L8" s="41"/>
-      <c r="M8" s="41"/>
-      <c r="N8" s="41"/>
-      <c r="O8" s="41"/>
+      <c r="C8" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="32"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="32"/>
+      <c r="J8" s="32"/>
+      <c r="K8" s="32"/>
+      <c r="L8" s="32"/>
+      <c r="M8" s="32"/>
+      <c r="N8" s="32"/>
+      <c r="O8" s="32"/>
       <c r="P8" s="2"/>
-      <c r="S8" s="47">
+      <c r="S8" s="38">
         <v>5</v>
       </c>
-      <c r="T8" s="46">
+      <c r="T8" s="37">
         <v>6</v>
       </c>
     </row>
     <row r="9" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="2"/>
-      <c r="C9" s="41" t="s">
-        <v>56</v>
-      </c>
-      <c r="D9" s="41"/>
-      <c r="E9" s="41"/>
-      <c r="F9" s="41"/>
-      <c r="G9" s="41"/>
-      <c r="H9" s="41"/>
-      <c r="I9" s="41"/>
-      <c r="J9" s="41"/>
-      <c r="K9" s="41"/>
-      <c r="L9" s="41"/>
-      <c r="M9" s="41"/>
-      <c r="N9" s="41"/>
-      <c r="O9" s="41"/>
+      <c r="C9" s="32" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
+      <c r="J9" s="32"/>
+      <c r="K9" s="32"/>
+      <c r="L9" s="32"/>
+      <c r="M9" s="32"/>
+      <c r="N9" s="32"/>
+      <c r="O9" s="32"/>
       <c r="P9" s="2"/>
-      <c r="S9" s="47">
+      <c r="S9" s="38">
         <v>6</v>
       </c>
-      <c r="T9" s="46">
+      <c r="T9" s="37">
         <v>5</v>
       </c>
     </row>
     <row r="10" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="2"/>
-      <c r="C10" s="41" t="s">
-        <v>57</v>
-      </c>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="41"/>
-      <c r="G10" s="41"/>
-      <c r="H10" s="41"/>
-      <c r="I10" s="41"/>
-      <c r="J10" s="41"/>
-      <c r="K10" s="41"/>
-      <c r="L10" s="41"/>
-      <c r="M10" s="41"/>
-      <c r="N10" s="41"/>
-      <c r="O10" s="41"/>
+      <c r="C10" s="32" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="32"/>
+      <c r="J10" s="32"/>
+      <c r="K10" s="32"/>
+      <c r="L10" s="32"/>
+      <c r="M10" s="32"/>
+      <c r="N10" s="32"/>
+      <c r="O10" s="32"/>
       <c r="P10" s="2"/>
-      <c r="S10" s="47">
+      <c r="S10" s="38">
         <v>7</v>
       </c>
-      <c r="T10" s="46">
+      <c r="T10" s="37">
         <v>4</v>
       </c>
     </row>
     <row r="11" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="2"/>
-      <c r="C11" s="41" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" s="41"/>
-      <c r="E11" s="41"/>
-      <c r="F11" s="41"/>
-      <c r="G11" s="41"/>
-      <c r="H11" s="41"/>
-      <c r="I11" s="41"/>
-      <c r="J11" s="41"/>
-      <c r="K11" s="41"/>
-      <c r="L11" s="41"/>
-      <c r="M11" s="41"/>
-      <c r="N11" s="41"/>
-      <c r="O11" s="41"/>
+      <c r="C11" s="32" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" s="32"/>
+      <c r="E11" s="32"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="32"/>
+      <c r="K11" s="32"/>
+      <c r="L11" s="32"/>
+      <c r="M11" s="32"/>
+      <c r="N11" s="32"/>
+      <c r="O11" s="32"/>
       <c r="P11" s="2"/>
-      <c r="S11" s="47">
+      <c r="S11" s="38">
         <v>8</v>
       </c>
-      <c r="T11" s="46">
+      <c r="T11" s="37">
         <v>3</v>
       </c>
     </row>
     <row r="12" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="2"/>
-      <c r="C12" s="41" t="s">
-        <v>59</v>
-      </c>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="41"/>
-      <c r="I12" s="41"/>
-      <c r="J12" s="41"/>
-      <c r="K12" s="41"/>
-      <c r="L12" s="41"/>
-      <c r="M12" s="41"/>
-      <c r="N12" s="41"/>
-      <c r="O12" s="41"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="32"/>
+      <c r="I12" s="32"/>
+      <c r="J12" s="32"/>
+      <c r="K12" s="32"/>
+      <c r="L12" s="32"/>
+      <c r="M12" s="32"/>
+      <c r="N12" s="32"/>
+      <c r="O12" s="32">
+        <v>2</v>
+      </c>
       <c r="P12" s="2"/>
-      <c r="S12" s="47">
+      <c r="S12" s="38">
         <v>9</v>
       </c>
-      <c r="T12" s="46">
+      <c r="T12" s="37">
         <v>2</v>
       </c>
     </row>
     <row r="13" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="2"/>
-      <c r="C13" s="41" t="s">
-        <v>60</v>
-      </c>
-      <c r="D13" s="41"/>
-      <c r="E13" s="41"/>
-      <c r="F13" s="41"/>
-      <c r="G13" s="41"/>
-      <c r="H13" s="41"/>
-      <c r="I13" s="41"/>
-      <c r="J13" s="41"/>
-      <c r="K13" s="41"/>
-      <c r="L13" s="41"/>
-      <c r="M13" s="41"/>
-      <c r="N13" s="41"/>
-      <c r="O13" s="41"/>
+      <c r="C13" s="32" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13" s="32"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="32"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="32"/>
+      <c r="K13" s="32"/>
+      <c r="L13" s="32"/>
+      <c r="M13" s="32"/>
+      <c r="N13" s="32"/>
+      <c r="O13" s="32"/>
       <c r="P13" s="2"/>
-      <c r="S13" s="47">
+      <c r="S13" s="38">
         <v>10</v>
       </c>
-      <c r="T13" s="46">
+      <c r="T13" s="37">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="2"/>
-      <c r="C14" s="41" t="s">
-        <v>61</v>
-      </c>
-      <c r="D14" s="41"/>
-      <c r="E14" s="41"/>
-      <c r="F14" s="41"/>
-      <c r="G14" s="41"/>
-      <c r="H14" s="41"/>
-      <c r="I14" s="41"/>
-      <c r="J14" s="41"/>
-      <c r="K14" s="41"/>
-      <c r="L14" s="41"/>
-      <c r="M14" s="41"/>
-      <c r="N14" s="41"/>
-      <c r="O14" s="41"/>
+      <c r="C14" s="32" t="s">
+        <v>59</v>
+      </c>
+      <c r="D14" s="32"/>
+      <c r="E14" s="32"/>
+      <c r="F14" s="32"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32"/>
+      <c r="I14" s="32"/>
+      <c r="J14" s="32"/>
+      <c r="K14" s="32"/>
+      <c r="L14" s="32"/>
+      <c r="M14" s="32"/>
+      <c r="N14" s="32"/>
+      <c r="O14" s="32"/>
       <c r="P14" s="2"/>
-      <c r="S14" s="47">
+      <c r="S14" s="38">
         <v>11</v>
       </c>
-      <c r="T14" s="46">
+      <c r="T14" s="37">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="2:20" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="2"/>
-      <c r="C15" s="40" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" s="42"/>
-      <c r="E15" s="42"/>
-      <c r="F15" s="42"/>
-      <c r="G15" s="42"/>
-      <c r="H15" s="42"/>
-      <c r="I15" s="42"/>
-      <c r="J15" s="42"/>
-      <c r="K15" s="42"/>
-      <c r="L15" s="42"/>
-      <c r="M15" s="42"/>
-      <c r="N15" s="42"/>
-      <c r="O15" s="42"/>
+      <c r="C15" s="31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="33">
+        <f>IFERROR(VLOOKUP(D5,S4:T15,2,0),0)+(D7+D8+D9+D10+D11+D12+D13+D14)*T16</f>
+        <v>0</v>
+      </c>
+      <c r="E15" s="33">
+        <f>IFERROR(VLOOKUP(E5,S4:T15,2,0),0)+(E7+E8+E9+E10+E11+E12+E13+E14)*T16</f>
+        <v>0</v>
+      </c>
+      <c r="F15" s="33">
+        <f>IFERROR(VLOOKUP(F5,S4:T15,2,0),0)+(F7+F8+F9+F10+F11+F12+F13+F14)*T16</f>
+        <v>0</v>
+      </c>
+      <c r="G15" s="33">
+        <f>IFERROR(VLOOKUP(G5,S4:T15,2,0),0)+(G7+G8+G9+G10+G11+G12+G13+G14)*T16</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="33">
+        <f>IFERROR(VLOOKUP(H5,S4:T15,2,0),0)+(H7+H8+H9+H10+H11+H12+H13+H14)*T16</f>
+        <v>0</v>
+      </c>
+      <c r="I15" s="33">
+        <f>IFERROR(VLOOKUP(I5,S4:T15,2,0),0)+(I7+I8+I9+I10+I11+I12+I13+I14)*T16</f>
+        <v>0</v>
+      </c>
+      <c r="J15" s="33">
+        <f>IFERROR(VLOOKUP(J5,S4:T15,2,0),0)+(J7+J8+J9+J10+J11+J12+J13+J14)*T16</f>
+        <v>0</v>
+      </c>
+      <c r="K15" s="33">
+        <f>IFERROR(VLOOKUP(K5,S4:T15,2,0),0)+(K7+K8+K9+K10+K11+K12+K13+K14)*T16</f>
+        <v>0</v>
+      </c>
+      <c r="L15" s="33">
+        <f>IFERROR(VLOOKUP(L5,S4:T15,2,0),0)+(L7+L8+L9+L10+L11+L12+L13+L14)*T16</f>
+        <v>0</v>
+      </c>
+      <c r="M15" s="33">
+        <f>IFERROR(VLOOKUP(M5,S4:T15,2,0),0)+(M7+M8+M9+M10+M11+M12+M13+M14)*T16</f>
+        <v>0</v>
+      </c>
+      <c r="N15" s="33">
+        <f>IFERROR(VLOOKUP(N5,S4:T15,2,0),0)+(N7+N8+N9+N10+N11+N12+N13+N14)*T16</f>
+        <v>0</v>
+      </c>
+      <c r="O15" s="33">
+        <f>IFERROR(VLOOKUP(O5,S4:T15,2,0),0)+(O7+O8+O9+O10+O11+O12+O13+O14)*T16</f>
+        <v>10</v>
+      </c>
       <c r="P15" s="2"/>
-      <c r="S15" s="47">
+      <c r="S15" s="38">
         <v>12</v>
       </c>
-      <c r="T15" s="46">
+      <c r="T15" s="37">
         <v>0</v>
       </c>
     </row>
@@ -5756,82 +5769,82 @@
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
       <c r="P16" s="2"/>
-      <c r="S16" s="48" t="s">
-        <v>12</v>
-      </c>
-      <c r="T16" s="49">
+      <c r="S16" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="T16" s="40">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="2:20" ht="26.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="2"/>
-      <c r="C17" s="39" t="s">
-        <v>13</v>
-      </c>
-      <c r="D17" s="39"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="39"/>
-      <c r="H17" s="39"/>
-      <c r="I17" s="39"/>
-      <c r="J17" s="39"/>
-      <c r="K17" s="39"/>
-      <c r="L17" s="39"/>
-      <c r="M17" s="39"/>
-      <c r="N17" s="39"/>
-      <c r="O17" s="39"/>
+      <c r="C17" s="79" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="79"/>
+      <c r="E17" s="79"/>
+      <c r="F17" s="79"/>
+      <c r="G17" s="79"/>
+      <c r="H17" s="79"/>
+      <c r="I17" s="79"/>
+      <c r="J17" s="79"/>
+      <c r="K17" s="79"/>
+      <c r="L17" s="79"/>
+      <c r="M17" s="79"/>
+      <c r="N17" s="79"/>
+      <c r="O17" s="79"/>
       <c r="P17" s="2"/>
     </row>
     <row r="18" spans="2:20" ht="26.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="2"/>
-      <c r="C18" s="40" t="s">
+      <c r="C18" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="D18" s="42" t="str">
+      <c r="D18" s="33" t="str">
         <f t="shared" ref="D18:O18" si="0">D4</f>
         <v>BERMUDA</v>
       </c>
-      <c r="E18" s="42" t="str">
+      <c r="E18" s="33" t="str">
         <f t="shared" si="0"/>
         <v>PURGATÓRIO</v>
       </c>
-      <c r="F18" s="42" t="str">
+      <c r="F18" s="33" t="str">
         <f t="shared" si="0"/>
         <v>KALAHARI</v>
       </c>
-      <c r="G18" s="42" t="str">
+      <c r="G18" s="33" t="str">
         <f t="shared" si="0"/>
         <v>NOVA TERRA</v>
       </c>
-      <c r="H18" s="42" t="str">
+      <c r="H18" s="33" t="str">
         <f t="shared" si="0"/>
         <v>ALPINE</v>
       </c>
-      <c r="I18" s="42" t="str">
+      <c r="I18" s="33" t="str">
         <f t="shared" si="0"/>
         <v>SOLARA</v>
       </c>
-      <c r="J18" s="42" t="str">
+      <c r="J18" s="33" t="str">
         <f t="shared" si="0"/>
         <v>BERMUDA</v>
       </c>
-      <c r="K18" s="42" t="str">
+      <c r="K18" s="33" t="str">
         <f t="shared" si="0"/>
         <v>PURGATÓRIO</v>
       </c>
-      <c r="L18" s="42" t="str">
+      <c r="L18" s="33" t="str">
         <f>L4</f>
         <v>KALAHARI</v>
       </c>
-      <c r="M18" s="42" t="str">
+      <c r="M18" s="33" t="str">
         <f>M4</f>
         <v>NOVA TERRA</v>
       </c>
-      <c r="N18" s="42" t="str">
+      <c r="N18" s="33" t="str">
         <f t="shared" si="0"/>
         <v>ALPINE</v>
       </c>
-      <c r="O18" s="42" t="str">
+      <c r="O18" s="33" t="str">
         <f t="shared" si="0"/>
         <v>SOLARA</v>
       </c>
@@ -5839,190 +5852,192 @@
     </row>
     <row r="19" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="2"/>
-      <c r="C19" s="42" t="str">
+      <c r="C19" s="33" t="str">
         <f t="shared" ref="C19:C26" si="1">C7</f>
         <v>JOGADOR 1</v>
       </c>
-      <c r="D19" s="41"/>
-      <c r="E19" s="41"/>
-      <c r="F19" s="41"/>
-      <c r="G19" s="41"/>
-      <c r="H19" s="41"/>
-      <c r="I19" s="41"/>
-      <c r="J19" s="41"/>
-      <c r="K19" s="41"/>
-      <c r="L19" s="41"/>
-      <c r="M19" s="41"/>
-      <c r="N19" s="41"/>
-      <c r="O19" s="41"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="32"/>
+      <c r="L19" s="32"/>
+      <c r="M19" s="32"/>
+      <c r="N19" s="32"/>
+      <c r="O19" s="32"/>
       <c r="P19" s="2"/>
-      <c r="S19" s="50" t="s">
-        <v>28</v>
-      </c>
-      <c r="T19" s="51"/>
+      <c r="S19" s="80" t="s">
+        <v>27</v>
+      </c>
+      <c r="T19" s="81"/>
     </row>
     <row r="20" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="2"/>
-      <c r="C20" s="42" t="str">
+      <c r="C20" s="33" t="str">
         <f t="shared" si="1"/>
         <v>JOGADOR 2</v>
       </c>
-      <c r="D20" s="41"/>
-      <c r="E20" s="41"/>
-      <c r="F20" s="41"/>
-      <c r="G20" s="41"/>
-      <c r="H20" s="41"/>
-      <c r="I20" s="41"/>
-      <c r="J20" s="41"/>
-      <c r="K20" s="41"/>
-      <c r="L20" s="41"/>
-      <c r="M20" s="41"/>
-      <c r="N20" s="41"/>
-      <c r="O20" s="41"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="32"/>
+      <c r="K20" s="32"/>
+      <c r="L20" s="32"/>
+      <c r="M20" s="32"/>
+      <c r="N20" s="32"/>
+      <c r="O20" s="32"/>
       <c r="P20" s="2"/>
-      <c r="S20" s="35" t="s">
+      <c r="S20" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="T20" s="36"/>
+      <c r="T20" s="83"/>
     </row>
     <row r="21" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="2"/>
-      <c r="C21" s="42" t="str">
+      <c r="C21" s="33" t="str">
         <f t="shared" si="1"/>
         <v>JOGADOR 3</v>
       </c>
-      <c r="D21" s="41"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="41"/>
-      <c r="I21" s="41"/>
-      <c r="J21" s="41"/>
-      <c r="K21" s="41"/>
-      <c r="L21" s="41"/>
-      <c r="M21" s="41"/>
-      <c r="N21" s="41"/>
-      <c r="O21" s="41"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="32"/>
+      <c r="L21" s="32"/>
+      <c r="M21" s="32"/>
+      <c r="N21" s="32"/>
+      <c r="O21" s="32"/>
       <c r="P21" s="2"/>
-      <c r="S21" s="31" t="s">
+      <c r="S21" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="T21" s="32"/>
+      <c r="T21" s="75"/>
     </row>
     <row r="22" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="2"/>
-      <c r="C22" s="42" t="str">
+      <c r="C22" s="33" t="str">
         <f t="shared" si="1"/>
         <v>JOGADOR 4</v>
       </c>
-      <c r="D22" s="41"/>
-      <c r="E22" s="41"/>
-      <c r="F22" s="41"/>
-      <c r="G22" s="41"/>
-      <c r="H22" s="41"/>
-      <c r="I22" s="41"/>
-      <c r="J22" s="41"/>
-      <c r="K22" s="41"/>
-      <c r="L22" s="41"/>
-      <c r="M22" s="41"/>
-      <c r="N22" s="41"/>
-      <c r="O22" s="41"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="32"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="32"/>
+      <c r="K22" s="32"/>
+      <c r="L22" s="32"/>
+      <c r="M22" s="32"/>
+      <c r="N22" s="32"/>
+      <c r="O22" s="32"/>
       <c r="P22" s="2"/>
-      <c r="S22" s="31" t="s">
+      <c r="S22" s="74" t="s">
         <v>6</v>
       </c>
-      <c r="T22" s="32"/>
+      <c r="T22" s="75"/>
     </row>
     <row r="23" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="2"/>
-      <c r="C23" s="42" t="str">
+      <c r="C23" s="33" t="str">
         <f t="shared" si="1"/>
         <v>RESERVA 1</v>
       </c>
-      <c r="D23" s="41"/>
-      <c r="E23" s="41"/>
-      <c r="F23" s="41"/>
-      <c r="G23" s="41"/>
-      <c r="H23" s="41"/>
-      <c r="I23" s="41"/>
-      <c r="J23" s="41"/>
-      <c r="K23" s="41"/>
-      <c r="L23" s="41"/>
-      <c r="M23" s="41"/>
-      <c r="N23" s="41"/>
-      <c r="O23" s="41"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="32"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="32"/>
+      <c r="J23" s="32"/>
+      <c r="K23" s="32"/>
+      <c r="L23" s="32"/>
+      <c r="M23" s="32"/>
+      <c r="N23" s="32"/>
+      <c r="O23" s="32">
+        <v>22</v>
+      </c>
       <c r="P23" s="2"/>
-      <c r="S23" s="31" t="s">
+      <c r="S23" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="T23" s="32"/>
+      <c r="T23" s="75"/>
     </row>
     <row r="24" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="2"/>
-      <c r="C24" s="42" t="str">
+      <c r="C24" s="33">
         <f t="shared" si="1"/>
-        <v>RESERVA 2</v>
-      </c>
-      <c r="D24" s="41"/>
-      <c r="E24" s="41"/>
-      <c r="F24" s="41"/>
-      <c r="G24" s="41"/>
-      <c r="H24" s="41"/>
-      <c r="I24" s="41"/>
-      <c r="J24" s="41"/>
-      <c r="K24" s="41"/>
-      <c r="L24" s="41"/>
-      <c r="M24" s="41"/>
-      <c r="N24" s="41"/>
-      <c r="O24" s="41"/>
+        <v>0</v>
+      </c>
+      <c r="D24" s="32"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
+      <c r="K24" s="32"/>
+      <c r="L24" s="32"/>
+      <c r="M24" s="32"/>
+      <c r="N24" s="32"/>
+      <c r="O24" s="32"/>
       <c r="P24" s="2"/>
-      <c r="S24" s="31" t="s">
+      <c r="S24" s="74" t="s">
         <v>8</v>
       </c>
-      <c r="T24" s="32"/>
+      <c r="T24" s="75"/>
     </row>
     <row r="25" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="2"/>
-      <c r="C25" s="42" t="str">
+      <c r="C25" s="33" t="str">
         <f t="shared" si="1"/>
         <v>RESERVA 3</v>
       </c>
-      <c r="D25" s="41"/>
-      <c r="E25" s="41"/>
-      <c r="F25" s="41"/>
-      <c r="G25" s="41"/>
-      <c r="H25" s="41"/>
-      <c r="I25" s="41"/>
-      <c r="J25" s="41"/>
-      <c r="K25" s="41"/>
-      <c r="L25" s="41"/>
-      <c r="M25" s="41"/>
-      <c r="N25" s="41"/>
-      <c r="O25" s="41"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="32"/>
+      <c r="K25" s="32"/>
+      <c r="L25" s="32"/>
+      <c r="M25" s="32"/>
+      <c r="N25" s="32"/>
+      <c r="O25" s="32"/>
       <c r="P25" s="2"/>
-      <c r="S25" s="37" t="s">
-        <v>53</v>
-      </c>
-      <c r="T25" s="38"/>
+      <c r="S25" s="84" t="s">
+        <v>52</v>
+      </c>
+      <c r="T25" s="85"/>
     </row>
     <row r="26" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="2"/>
-      <c r="C26" s="42" t="str">
+      <c r="C26" s="33" t="str">
         <f t="shared" si="1"/>
         <v>RESERVA 4</v>
       </c>
-      <c r="D26" s="41"/>
-      <c r="E26" s="41"/>
-      <c r="F26" s="41"/>
-      <c r="G26" s="41"/>
-      <c r="H26" s="41"/>
-      <c r="I26" s="41"/>
-      <c r="J26" s="41"/>
-      <c r="K26" s="41"/>
-      <c r="L26" s="41"/>
-      <c r="M26" s="41"/>
-      <c r="N26" s="41"/>
-      <c r="O26" s="41"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="32"/>
+      <c r="F26" s="32"/>
+      <c r="G26" s="32"/>
+      <c r="H26" s="32"/>
+      <c r="I26" s="32"/>
+      <c r="J26" s="32"/>
+      <c r="K26" s="32"/>
+      <c r="L26" s="32"/>
+      <c r="M26" s="32"/>
+      <c r="N26" s="32"/>
+      <c r="O26" s="32"/>
       <c r="P26" s="2"/>
     </row>
     <row r="27" spans="2:20" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6044,73 +6059,73 @@
     </row>
     <row r="28" spans="2:20" ht="26.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B28" s="2"/>
-      <c r="C28" s="39" t="s">
-        <v>14</v>
-      </c>
-      <c r="D28" s="39"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="39"/>
-      <c r="G28" s="39"/>
-      <c r="H28" s="39"/>
-      <c r="I28" s="39"/>
-      <c r="J28" s="39"/>
-      <c r="K28" s="39"/>
-      <c r="L28" s="39"/>
-      <c r="M28" s="39"/>
-      <c r="N28" s="39"/>
-      <c r="O28" s="39"/>
+      <c r="C28" s="79" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="79"/>
+      <c r="E28" s="79"/>
+      <c r="F28" s="79"/>
+      <c r="G28" s="79"/>
+      <c r="H28" s="79"/>
+      <c r="I28" s="79"/>
+      <c r="J28" s="79"/>
+      <c r="K28" s="79"/>
+      <c r="L28" s="79"/>
+      <c r="M28" s="79"/>
+      <c r="N28" s="79"/>
+      <c r="O28" s="79"/>
       <c r="P28" s="2"/>
     </row>
     <row r="29" spans="2:20" ht="26.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="2"/>
-      <c r="C29" s="40" t="s">
+      <c r="C29" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="D29" s="42" t="str">
+      <c r="D29" s="33" t="str">
         <f t="shared" ref="D29:O29" si="2">D4</f>
         <v>BERMUDA</v>
       </c>
-      <c r="E29" s="42" t="str">
+      <c r="E29" s="33" t="str">
         <f t="shared" si="2"/>
         <v>PURGATÓRIO</v>
       </c>
-      <c r="F29" s="42" t="str">
+      <c r="F29" s="33" t="str">
         <f t="shared" si="2"/>
         <v>KALAHARI</v>
       </c>
-      <c r="G29" s="42" t="str">
+      <c r="G29" s="33" t="str">
         <f t="shared" si="2"/>
         <v>NOVA TERRA</v>
       </c>
-      <c r="H29" s="42" t="str">
+      <c r="H29" s="33" t="str">
         <f t="shared" si="2"/>
         <v>ALPINE</v>
       </c>
-      <c r="I29" s="42" t="str">
+      <c r="I29" s="33" t="str">
         <f t="shared" si="2"/>
         <v>SOLARA</v>
       </c>
-      <c r="J29" s="42" t="str">
+      <c r="J29" s="33" t="str">
         <f t="shared" si="2"/>
         <v>BERMUDA</v>
       </c>
-      <c r="K29" s="42" t="str">
+      <c r="K29" s="33" t="str">
         <f t="shared" si="2"/>
         <v>PURGATÓRIO</v>
       </c>
-      <c r="L29" s="42" t="str">
+      <c r="L29" s="33" t="str">
         <f>L4</f>
         <v>KALAHARI</v>
       </c>
-      <c r="M29" s="42" t="str">
+      <c r="M29" s="33" t="str">
         <f>M4</f>
         <v>NOVA TERRA</v>
       </c>
-      <c r="N29" s="42" t="str">
+      <c r="N29" s="33" t="str">
         <f t="shared" si="2"/>
         <v>ALPINE</v>
       </c>
-      <c r="O29" s="42" t="str">
+      <c r="O29" s="33" t="str">
         <f t="shared" si="2"/>
         <v>SOLARA</v>
       </c>
@@ -6118,162 +6133,162 @@
     </row>
     <row r="30" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B30" s="2"/>
-      <c r="C30" s="42" t="str">
+      <c r="C30" s="33" t="str">
         <f t="shared" ref="C30:C37" si="3">C7</f>
         <v>JOGADOR 1</v>
       </c>
-      <c r="D30" s="43"/>
-      <c r="E30" s="43"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="43"/>
-      <c r="H30" s="43"/>
-      <c r="I30" s="43"/>
-      <c r="J30" s="43"/>
-      <c r="K30" s="43"/>
-      <c r="L30" s="43"/>
-      <c r="M30" s="43"/>
-      <c r="N30" s="43"/>
-      <c r="O30" s="43"/>
+      <c r="D30" s="34"/>
+      <c r="E30" s="34"/>
+      <c r="F30" s="34"/>
+      <c r="G30" s="34"/>
+      <c r="H30" s="34"/>
+      <c r="I30" s="34"/>
+      <c r="J30" s="34"/>
+      <c r="K30" s="34"/>
+      <c r="L30" s="34"/>
+      <c r="M30" s="34"/>
+      <c r="N30" s="34"/>
+      <c r="O30" s="34"/>
       <c r="P30" s="3"/>
     </row>
     <row r="31" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="2"/>
-      <c r="C31" s="42" t="str">
+      <c r="C31" s="33" t="str">
         <f t="shared" si="3"/>
         <v>JOGADOR 2</v>
       </c>
-      <c r="D31" s="43"/>
-      <c r="E31" s="43"/>
-      <c r="F31" s="43"/>
-      <c r="G31" s="43"/>
-      <c r="H31" s="43"/>
-      <c r="I31" s="43"/>
-      <c r="J31" s="43"/>
-      <c r="K31" s="43"/>
-      <c r="L31" s="43"/>
-      <c r="M31" s="43"/>
-      <c r="N31" s="43"/>
-      <c r="O31" s="43"/>
+      <c r="D31" s="34"/>
+      <c r="E31" s="34"/>
+      <c r="F31" s="34"/>
+      <c r="G31" s="34"/>
+      <c r="H31" s="34"/>
+      <c r="I31" s="34"/>
+      <c r="J31" s="34"/>
+      <c r="K31" s="34"/>
+      <c r="L31" s="34"/>
+      <c r="M31" s="34"/>
+      <c r="N31" s="34"/>
+      <c r="O31" s="34"/>
       <c r="P31" s="2"/>
     </row>
     <row r="32" spans="2:20" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="2"/>
-      <c r="C32" s="42" t="str">
+      <c r="C32" s="33" t="str">
         <f t="shared" si="3"/>
         <v>JOGADOR 3</v>
       </c>
-      <c r="D32" s="43"/>
-      <c r="E32" s="43"/>
-      <c r="F32" s="43"/>
-      <c r="G32" s="43"/>
-      <c r="H32" s="43"/>
-      <c r="I32" s="43"/>
-      <c r="J32" s="43"/>
-      <c r="K32" s="43"/>
-      <c r="L32" s="43"/>
-      <c r="M32" s="43"/>
-      <c r="N32" s="43"/>
-      <c r="O32" s="43"/>
+      <c r="D32" s="34"/>
+      <c r="E32" s="34"/>
+      <c r="F32" s="34"/>
+      <c r="G32" s="34"/>
+      <c r="H32" s="34"/>
+      <c r="I32" s="34"/>
+      <c r="J32" s="34"/>
+      <c r="K32" s="34"/>
+      <c r="L32" s="34"/>
+      <c r="M32" s="34"/>
+      <c r="N32" s="34"/>
+      <c r="O32" s="34"/>
       <c r="P32" s="2"/>
     </row>
     <row r="33" spans="2:19" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="2"/>
-      <c r="C33" s="42" t="str">
+      <c r="C33" s="33" t="str">
         <f t="shared" si="3"/>
         <v>JOGADOR 4</v>
       </c>
-      <c r="D33" s="43"/>
-      <c r="E33" s="43"/>
-      <c r="F33" s="43"/>
-      <c r="G33" s="43"/>
-      <c r="H33" s="43"/>
-      <c r="I33" s="43"/>
-      <c r="J33" s="43"/>
-      <c r="K33" s="43"/>
-      <c r="L33" s="43"/>
-      <c r="M33" s="43"/>
-      <c r="N33" s="43"/>
-      <c r="O33" s="43"/>
+      <c r="D33" s="34"/>
+      <c r="E33" s="34"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="34"/>
+      <c r="H33" s="34"/>
+      <c r="I33" s="34"/>
+      <c r="J33" s="34"/>
+      <c r="K33" s="34"/>
+      <c r="L33" s="34"/>
+      <c r="M33" s="34"/>
+      <c r="N33" s="34"/>
+      <c r="O33" s="34"/>
       <c r="P33" s="2"/>
     </row>
     <row r="34" spans="2:19" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B34" s="2"/>
-      <c r="C34" s="42" t="str">
+      <c r="C34" s="33" t="str">
         <f t="shared" si="3"/>
         <v>RESERVA 1</v>
       </c>
-      <c r="D34" s="43"/>
-      <c r="E34" s="43"/>
-      <c r="F34" s="43"/>
-      <c r="G34" s="43"/>
-      <c r="H34" s="43"/>
-      <c r="I34" s="43"/>
-      <c r="J34" s="43"/>
-      <c r="K34" s="43"/>
-      <c r="L34" s="43"/>
-      <c r="M34" s="43"/>
-      <c r="N34" s="43"/>
-      <c r="O34" s="43"/>
+      <c r="D34" s="34"/>
+      <c r="E34" s="34"/>
+      <c r="F34" s="34"/>
+      <c r="G34" s="34"/>
+      <c r="H34" s="34"/>
+      <c r="I34" s="34"/>
+      <c r="J34" s="34"/>
+      <c r="K34" s="34"/>
+      <c r="L34" s="34"/>
+      <c r="M34" s="34"/>
+      <c r="N34" s="34"/>
+      <c r="O34" s="34"/>
       <c r="P34" s="2"/>
     </row>
     <row r="35" spans="2:19" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B35" s="2"/>
-      <c r="C35" s="42" t="str">
+      <c r="C35" s="33">
         <f t="shared" si="3"/>
-        <v>RESERVA 2</v>
-      </c>
-      <c r="D35" s="43"/>
-      <c r="E35" s="43"/>
-      <c r="F35" s="43"/>
-      <c r="G35" s="43"/>
-      <c r="H35" s="43"/>
-      <c r="I35" s="43"/>
-      <c r="J35" s="43"/>
-      <c r="K35" s="43"/>
-      <c r="L35" s="43"/>
-      <c r="M35" s="43"/>
-      <c r="N35" s="43"/>
-      <c r="O35" s="43"/>
+        <v>0</v>
+      </c>
+      <c r="D35" s="34"/>
+      <c r="E35" s="34"/>
+      <c r="F35" s="34"/>
+      <c r="G35" s="34"/>
+      <c r="H35" s="34"/>
+      <c r="I35" s="34"/>
+      <c r="J35" s="34"/>
+      <c r="K35" s="34"/>
+      <c r="L35" s="34"/>
+      <c r="M35" s="34"/>
+      <c r="N35" s="34"/>
+      <c r="O35" s="34"/>
       <c r="P35" s="2"/>
     </row>
     <row r="36" spans="2:19" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="2"/>
-      <c r="C36" s="42" t="str">
+      <c r="C36" s="33" t="str">
         <f t="shared" si="3"/>
         <v>RESERVA 3</v>
       </c>
-      <c r="D36" s="43"/>
-      <c r="E36" s="43"/>
-      <c r="F36" s="43"/>
-      <c r="G36" s="43"/>
-      <c r="H36" s="43"/>
-      <c r="I36" s="43"/>
-      <c r="J36" s="43"/>
-      <c r="K36" s="43"/>
-      <c r="L36" s="43"/>
-      <c r="M36" s="43"/>
-      <c r="N36" s="43"/>
-      <c r="O36" s="43"/>
+      <c r="D36" s="34"/>
+      <c r="E36" s="34"/>
+      <c r="F36" s="34"/>
+      <c r="G36" s="34"/>
+      <c r="H36" s="34"/>
+      <c r="I36" s="34"/>
+      <c r="J36" s="34"/>
+      <c r="K36" s="34"/>
+      <c r="L36" s="34"/>
+      <c r="M36" s="34"/>
+      <c r="N36" s="34"/>
+      <c r="O36" s="34"/>
       <c r="P36" s="2"/>
     </row>
     <row r="37" spans="2:19" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B37" s="2"/>
-      <c r="C37" s="42" t="str">
+      <c r="C37" s="33" t="str">
         <f t="shared" si="3"/>
         <v>RESERVA 4</v>
       </c>
-      <c r="D37" s="43"/>
-      <c r="E37" s="43"/>
-      <c r="F37" s="43"/>
-      <c r="G37" s="43"/>
-      <c r="H37" s="43"/>
-      <c r="I37" s="43"/>
-      <c r="J37" s="43"/>
-      <c r="K37" s="43"/>
-      <c r="L37" s="43"/>
-      <c r="M37" s="43"/>
-      <c r="N37" s="43"/>
-      <c r="O37" s="43"/>
+      <c r="D37" s="34"/>
+      <c r="E37" s="34"/>
+      <c r="F37" s="34"/>
+      <c r="G37" s="34"/>
+      <c r="H37" s="34"/>
+      <c r="I37" s="34"/>
+      <c r="J37" s="34"/>
+      <c r="K37" s="34"/>
+      <c r="L37" s="34"/>
+      <c r="M37" s="34"/>
+      <c r="N37" s="34"/>
+      <c r="O37" s="34"/>
       <c r="P37" s="2"/>
     </row>
     <row r="38" spans="2:19" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6295,74 +6310,74 @@
     </row>
     <row r="39" spans="2:19" s="5" customFormat="1" ht="26.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B39" s="4"/>
-      <c r="C39" s="39" t="s">
-        <v>15</v>
-      </c>
-      <c r="D39" s="39"/>
-      <c r="E39" s="39"/>
-      <c r="F39" s="39"/>
-      <c r="G39" s="39"/>
-      <c r="H39" s="39"/>
-      <c r="I39" s="39"/>
-      <c r="J39" s="39"/>
-      <c r="K39" s="39"/>
-      <c r="L39" s="39"/>
-      <c r="M39" s="39"/>
-      <c r="N39" s="39"/>
-      <c r="O39" s="39"/>
+      <c r="C39" s="79" t="s">
+        <v>14</v>
+      </c>
+      <c r="D39" s="79"/>
+      <c r="E39" s="79"/>
+      <c r="F39" s="79"/>
+      <c r="G39" s="79"/>
+      <c r="H39" s="79"/>
+      <c r="I39" s="79"/>
+      <c r="J39" s="79"/>
+      <c r="K39" s="79"/>
+      <c r="L39" s="79"/>
+      <c r="M39" s="79"/>
+      <c r="N39" s="79"/>
+      <c r="O39" s="79"/>
       <c r="P39" s="4"/>
       <c r="S39" s="1"/>
     </row>
     <row r="40" spans="2:19" ht="26.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B40" s="2"/>
-      <c r="C40" s="40" t="s">
+      <c r="C40" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="D40" s="42" t="str">
+      <c r="D40" s="33" t="str">
         <f t="shared" ref="D40:O40" si="4">D4</f>
         <v>BERMUDA</v>
       </c>
-      <c r="E40" s="42" t="str">
+      <c r="E40" s="33" t="str">
         <f t="shared" si="4"/>
         <v>PURGATÓRIO</v>
       </c>
-      <c r="F40" s="42" t="str">
+      <c r="F40" s="33" t="str">
         <f t="shared" si="4"/>
         <v>KALAHARI</v>
       </c>
-      <c r="G40" s="42" t="str">
+      <c r="G40" s="33" t="str">
         <f t="shared" si="4"/>
         <v>NOVA TERRA</v>
       </c>
-      <c r="H40" s="42" t="str">
+      <c r="H40" s="33" t="str">
         <f t="shared" si="4"/>
         <v>ALPINE</v>
       </c>
-      <c r="I40" s="42" t="str">
+      <c r="I40" s="33" t="str">
         <f t="shared" si="4"/>
         <v>SOLARA</v>
       </c>
-      <c r="J40" s="42" t="str">
+      <c r="J40" s="33" t="str">
         <f t="shared" si="4"/>
         <v>BERMUDA</v>
       </c>
-      <c r="K40" s="42" t="str">
+      <c r="K40" s="33" t="str">
         <f t="shared" si="4"/>
         <v>PURGATÓRIO</v>
       </c>
-      <c r="L40" s="42" t="str">
+      <c r="L40" s="33" t="str">
         <f>L4</f>
         <v>KALAHARI</v>
       </c>
-      <c r="M40" s="42" t="str">
+      <c r="M40" s="33" t="str">
         <f>M4</f>
         <v>NOVA TERRA</v>
       </c>
-      <c r="N40" s="42" t="str">
+      <c r="N40" s="33" t="str">
         <f t="shared" si="4"/>
         <v>ALPINE</v>
       </c>
-      <c r="O40" s="42" t="str">
+      <c r="O40" s="33" t="str">
         <f t="shared" si="4"/>
         <v>SOLARA</v>
       </c>
@@ -6370,162 +6385,162 @@
     </row>
     <row r="41" spans="2:19" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B41" s="2"/>
-      <c r="C41" s="42" t="str">
+      <c r="C41" s="33" t="str">
         <f t="shared" ref="C41:C48" si="5">C7</f>
         <v>JOGADOR 1</v>
       </c>
-      <c r="D41" s="41"/>
-      <c r="E41" s="41"/>
-      <c r="F41" s="41"/>
-      <c r="G41" s="41"/>
-      <c r="H41" s="41"/>
-      <c r="I41" s="41"/>
-      <c r="J41" s="41"/>
-      <c r="K41" s="41"/>
-      <c r="L41" s="41"/>
-      <c r="M41" s="41"/>
-      <c r="N41" s="41"/>
-      <c r="O41" s="41"/>
+      <c r="D41" s="32"/>
+      <c r="E41" s="32"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="32"/>
+      <c r="H41" s="32"/>
+      <c r="I41" s="32"/>
+      <c r="J41" s="32"/>
+      <c r="K41" s="32"/>
+      <c r="L41" s="32"/>
+      <c r="M41" s="32"/>
+      <c r="N41" s="32"/>
+      <c r="O41" s="32"/>
       <c r="P41" s="2"/>
     </row>
     <row r="42" spans="2:19" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B42" s="2"/>
-      <c r="C42" s="42" t="str">
+      <c r="C42" s="33" t="str">
         <f t="shared" si="5"/>
         <v>JOGADOR 2</v>
       </c>
-      <c r="D42" s="41"/>
-      <c r="E42" s="41"/>
-      <c r="F42" s="41"/>
-      <c r="G42" s="41"/>
-      <c r="H42" s="41"/>
-      <c r="I42" s="41"/>
-      <c r="J42" s="41"/>
-      <c r="K42" s="41"/>
-      <c r="L42" s="41"/>
-      <c r="M42" s="41"/>
-      <c r="N42" s="41"/>
-      <c r="O42" s="41"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="32"/>
+      <c r="F42" s="32"/>
+      <c r="G42" s="32"/>
+      <c r="H42" s="32"/>
+      <c r="I42" s="32"/>
+      <c r="J42" s="32"/>
+      <c r="K42" s="32"/>
+      <c r="L42" s="32"/>
+      <c r="M42" s="32"/>
+      <c r="N42" s="32"/>
+      <c r="O42" s="32"/>
       <c r="P42" s="6"/>
     </row>
     <row r="43" spans="2:19" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B43" s="2"/>
-      <c r="C43" s="42" t="str">
+      <c r="C43" s="33" t="str">
         <f t="shared" si="5"/>
         <v>JOGADOR 3</v>
       </c>
-      <c r="D43" s="41"/>
-      <c r="E43" s="41"/>
-      <c r="F43" s="41"/>
-      <c r="G43" s="41"/>
-      <c r="H43" s="41"/>
-      <c r="I43" s="41"/>
-      <c r="J43" s="41"/>
-      <c r="K43" s="41"/>
-      <c r="L43" s="41"/>
-      <c r="M43" s="41"/>
-      <c r="N43" s="41"/>
-      <c r="O43" s="41"/>
+      <c r="D43" s="32"/>
+      <c r="E43" s="32"/>
+      <c r="F43" s="32"/>
+      <c r="G43" s="32"/>
+      <c r="H43" s="32"/>
+      <c r="I43" s="32"/>
+      <c r="J43" s="32"/>
+      <c r="K43" s="32"/>
+      <c r="L43" s="32"/>
+      <c r="M43" s="32"/>
+      <c r="N43" s="32"/>
+      <c r="O43" s="32"/>
       <c r="P43" s="2"/>
     </row>
     <row r="44" spans="2:19" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B44" s="2"/>
-      <c r="C44" s="42" t="str">
+      <c r="C44" s="33" t="str">
         <f t="shared" si="5"/>
         <v>JOGADOR 4</v>
       </c>
-      <c r="D44" s="41"/>
-      <c r="E44" s="41"/>
-      <c r="F44" s="41"/>
-      <c r="G44" s="41"/>
-      <c r="H44" s="41"/>
-      <c r="I44" s="41"/>
-      <c r="J44" s="41"/>
-      <c r="K44" s="41"/>
-      <c r="L44" s="41"/>
-      <c r="M44" s="41"/>
-      <c r="N44" s="41"/>
-      <c r="O44" s="41"/>
+      <c r="D44" s="32"/>
+      <c r="E44" s="32"/>
+      <c r="F44" s="32"/>
+      <c r="G44" s="32"/>
+      <c r="H44" s="32"/>
+      <c r="I44" s="32"/>
+      <c r="J44" s="32"/>
+      <c r="K44" s="32"/>
+      <c r="L44" s="32"/>
+      <c r="M44" s="32"/>
+      <c r="N44" s="32"/>
+      <c r="O44" s="32"/>
       <c r="P44" s="2"/>
     </row>
     <row r="45" spans="2:19" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B45" s="2"/>
-      <c r="C45" s="42" t="str">
+      <c r="C45" s="33" t="str">
         <f t="shared" si="5"/>
         <v>RESERVA 1</v>
       </c>
-      <c r="D45" s="41"/>
-      <c r="E45" s="41"/>
-      <c r="F45" s="41"/>
-      <c r="G45" s="41"/>
-      <c r="H45" s="41"/>
-      <c r="I45" s="41"/>
-      <c r="J45" s="41"/>
-      <c r="K45" s="41"/>
-      <c r="L45" s="41"/>
-      <c r="M45" s="41"/>
-      <c r="N45" s="41"/>
-      <c r="O45" s="41"/>
+      <c r="D45" s="32"/>
+      <c r="E45" s="32"/>
+      <c r="F45" s="32"/>
+      <c r="G45" s="32"/>
+      <c r="H45" s="32"/>
+      <c r="I45" s="32"/>
+      <c r="J45" s="32"/>
+      <c r="K45" s="32"/>
+      <c r="L45" s="32"/>
+      <c r="M45" s="32"/>
+      <c r="N45" s="32"/>
+      <c r="O45" s="32"/>
       <c r="P45" s="2"/>
     </row>
     <row r="46" spans="2:19" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B46" s="2"/>
-      <c r="C46" s="42" t="str">
+      <c r="C46" s="33">
         <f t="shared" si="5"/>
-        <v>RESERVA 2</v>
-      </c>
-      <c r="D46" s="41"/>
-      <c r="E46" s="41"/>
-      <c r="F46" s="41"/>
-      <c r="G46" s="41"/>
-      <c r="H46" s="41"/>
-      <c r="I46" s="41"/>
-      <c r="J46" s="41"/>
-      <c r="K46" s="41"/>
-      <c r="L46" s="41"/>
-      <c r="M46" s="41"/>
-      <c r="N46" s="41"/>
-      <c r="O46" s="41"/>
+        <v>0</v>
+      </c>
+      <c r="D46" s="32"/>
+      <c r="E46" s="32"/>
+      <c r="F46" s="32"/>
+      <c r="G46" s="32"/>
+      <c r="H46" s="32"/>
+      <c r="I46" s="32"/>
+      <c r="J46" s="32"/>
+      <c r="K46" s="32"/>
+      <c r="L46" s="32"/>
+      <c r="M46" s="32"/>
+      <c r="N46" s="32"/>
+      <c r="O46" s="32"/>
       <c r="P46" s="2"/>
     </row>
     <row r="47" spans="2:19" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B47" s="2"/>
-      <c r="C47" s="42" t="str">
+      <c r="C47" s="33" t="str">
         <f t="shared" si="5"/>
         <v>RESERVA 3</v>
       </c>
-      <c r="D47" s="41"/>
-      <c r="E47" s="41"/>
-      <c r="F47" s="41"/>
-      <c r="G47" s="41"/>
-      <c r="H47" s="41"/>
-      <c r="I47" s="41"/>
-      <c r="J47" s="41"/>
-      <c r="K47" s="41"/>
-      <c r="L47" s="41"/>
-      <c r="M47" s="41"/>
-      <c r="N47" s="41"/>
-      <c r="O47" s="41"/>
+      <c r="D47" s="32"/>
+      <c r="E47" s="32"/>
+      <c r="F47" s="32"/>
+      <c r="G47" s="32"/>
+      <c r="H47" s="32"/>
+      <c r="I47" s="32"/>
+      <c r="J47" s="32"/>
+      <c r="K47" s="32"/>
+      <c r="L47" s="32"/>
+      <c r="M47" s="32"/>
+      <c r="N47" s="32"/>
+      <c r="O47" s="32"/>
       <c r="P47" s="2"/>
     </row>
     <row r="48" spans="2:19" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B48" s="2"/>
-      <c r="C48" s="42" t="str">
+      <c r="C48" s="33" t="str">
         <f t="shared" si="5"/>
         <v>RESERVA 4</v>
       </c>
-      <c r="D48" s="41"/>
-      <c r="E48" s="41"/>
-      <c r="F48" s="41"/>
-      <c r="G48" s="41"/>
-      <c r="H48" s="41"/>
-      <c r="I48" s="41"/>
-      <c r="J48" s="41"/>
-      <c r="K48" s="41"/>
-      <c r="L48" s="41"/>
-      <c r="M48" s="41"/>
-      <c r="N48" s="41"/>
-      <c r="O48" s="41"/>
+      <c r="D48" s="32"/>
+      <c r="E48" s="32"/>
+      <c r="F48" s="32"/>
+      <c r="G48" s="32"/>
+      <c r="H48" s="32"/>
+      <c r="I48" s="32"/>
+      <c r="J48" s="32"/>
+      <c r="K48" s="32"/>
+      <c r="L48" s="32"/>
+      <c r="M48" s="32"/>
+      <c r="N48" s="32"/>
+      <c r="O48" s="32"/>
       <c r="P48" s="2"/>
     </row>
     <row r="49" spans="2:16" ht="27.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
@@ -6546,7 +6561,7 @@
       <c r="P49" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="iE7uS31bcY7eUHMrVMvt5ssaMkxv/N5wBdsf6DPEjTjt8Z2vKT0laU6M72j1lCz+WlL0YVjYn6J0MOEtk0zzUw==" saltValue="Py3R8VaHXkRl7FVOYhfLZQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="e43MjUtwyTroMGd4rVitw8EWS50It7nZdaSiBmGYDO9LQ8mnLTqgFqOXe93CPY4DLUX4Vm2m2sxegke16bq0fg==" saltValue="ZItDNS0NRzoGTgHlE1LdTA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="12">
     <mergeCell ref="S24:T24"/>
     <mergeCell ref="C3:O3"/>
@@ -6566,7 +6581,7 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="AVISO!" prompt="Para  funcionar corretamente digite o horário da seguinte forma:_x000a_00:00:00_x000a_hora:minuto:segundo_x000a_" sqref="D30:O37" xr:uid="{A51CE2DC-053A-4DAF-89F8-F67C966A8D9E}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="AVISO!" prompt="Altere a pontuação aqui se for necessário._x000a_" sqref="T4:T16" xr:uid="{02DC377D-17D3-496C-8F05-131A34407121}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="S20:T25" xr:uid="{9AF71F29-72B0-4BAE-844A-48620EC2F20F}">
-      <formula1>$S$20:$S$25</formula1>
+      <formula1>"BERMUDA,PURGATÓRIO,KALAHARI,NOVA TERRA,ALPINE,SOLARA"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D4:O4" xr:uid="{EAE3FBFF-9AAC-4830-8D40-B0327DB42522}">
       <formula1>$D$4:$O$4</formula1>
@@ -6595,355 +6610,355 @@
     <col min="15" max="21" width="9.140625" style="1" hidden="1" customWidth="1"/>
     <col min="22" max="22" width="11.28515625" style="1" hidden="1" customWidth="1"/>
     <col min="23" max="30" width="9.140625" style="1" hidden="1" customWidth="1"/>
-    <col min="31" max="31" width="10.42578125" style="1" hidden="1" customWidth="1"/>
+    <col min="31" max="31" width="10.28515625" style="1" hidden="1" customWidth="1"/>
     <col min="32" max="33" width="0" style="1" hidden="1" customWidth="1"/>
     <col min="34" max="16384" width="9.140625" style="1" hidden="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:33" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="2:33" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="55" t="s">
+      <c r="C3" s="89" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="52" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" s="53"/>
-      <c r="F3" s="53"/>
-      <c r="G3" s="53"/>
-      <c r="H3" s="53"/>
-      <c r="I3" s="53"/>
-      <c r="J3" s="53"/>
-      <c r="K3" s="54"/>
+      <c r="D3" s="86" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="87"/>
+      <c r="F3" s="87"/>
+      <c r="G3" s="87"/>
+      <c r="H3" s="87"/>
+      <c r="I3" s="87"/>
+      <c r="J3" s="87"/>
+      <c r="K3" s="88"/>
     </row>
     <row r="4" spans="2:33" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="7"/>
-      <c r="C4" s="56"/>
-      <c r="D4" s="57" t="s">
+      <c r="C4" s="90"/>
+      <c r="D4" s="41" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="58" t="s">
+      <c r="F4" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="58" t="s">
+      <c r="G4" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="58" t="s">
+      <c r="H4" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="H4" s="58" t="s">
+      <c r="I4" s="42" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="58" t="s">
-        <v>14</v>
-      </c>
-      <c r="J4" s="58" t="s">
+      <c r="K4" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="K4" s="59" t="s">
-        <v>22</v>
-      </c>
     </row>
     <row r="5" spans="2:33" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="74" t="str">
+      <c r="C5" s="58" t="str">
         <f>'DADOS DO TIME'!C7</f>
         <v>JOGADOR 1</v>
       </c>
-      <c r="D5" s="60">
+      <c r="D5" s="44">
         <f>SUM('DADOS DO TIME'!D7:O7)</f>
         <v>0</v>
       </c>
-      <c r="E5" s="61">
+      <c r="E5" s="45">
         <f>IFERROR(D5/K5,0)</f>
         <v>0</v>
       </c>
-      <c r="F5" s="62">
+      <c r="F5" s="46">
         <f>SUM('DADOS DO TIME'!D19:O19)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="62">
+      <c r="G5" s="46">
         <f>'DADOS DO TIME'!D41+'DADOS DO TIME'!E41+'DADOS DO TIME'!F41+'DADOS DO TIME'!G41+'DADOS DO TIME'!H41+'DADOS DO TIME'!I41+'DADOS DO TIME'!J41+'DADOS DO TIME'!K41+'DADOS DO TIME'!N41+'DADOS DO TIME'!O41</f>
         <v>0</v>
       </c>
-      <c r="H5" s="61">
+      <c r="H5" s="45">
         <f>IFERROR(AVERAGE('DADOS DO TIME'!D41,'DADOS DO TIME'!E41,'DADOS DO TIME'!F41,'DADOS DO TIME'!G41,'DADOS DO TIME'!H41,'DADOS DO TIME'!I41,'DADOS DO TIME'!J41,'DADOS DO TIME'!K41,'DADOS DO TIME'!N41,'DADOS DO TIME'!O41),0)</f>
         <v>0</v>
       </c>
-      <c r="I5" s="63">
+      <c r="I5" s="47">
         <f>SUM('DADOS DO TIME'!D30:O30)</f>
         <v>0</v>
       </c>
-      <c r="J5" s="63">
+      <c r="J5" s="47">
         <f>IFERROR(AVERAGE('DADOS DO TIME'!D30,'DADOS DO TIME'!E30,'DADOS DO TIME'!F30,'DADOS DO TIME'!G30,'DADOS DO TIME'!H30,'DADOS DO TIME'!I30,'DADOS DO TIME'!J30,'DADOS DO TIME'!K30,'DADOS DO TIME'!N30,'DADOS DO TIME'!O30),0)</f>
         <v>0</v>
       </c>
-      <c r="K5" s="64">
+      <c r="K5" s="48">
         <f>COUNT('DADOS DO TIME'!D7,'DADOS DO TIME'!E7,'DADOS DO TIME'!F7,'DADOS DO TIME'!G7,'DADOS DO TIME'!H7,'DADOS DO TIME'!I7,'DADOS DO TIME'!J7,'DADOS DO TIME'!K7,'DADOS DO TIME'!N7,'DADOS DO TIME'!O7)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="2:33" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="75" t="str">
+      <c r="C6" s="59" t="str">
         <f>'DADOS DO TIME'!C8</f>
         <v>JOGADOR 2</v>
       </c>
-      <c r="D6" s="65">
+      <c r="D6" s="49">
         <f>SUM('DADOS DO TIME'!D8:O8)</f>
         <v>0</v>
       </c>
-      <c r="E6" s="66">
+      <c r="E6" s="50">
         <f t="shared" ref="E6:E12" si="0">IFERROR(D6/K6,0)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="42">
+      <c r="F6" s="33">
         <f>SUM('DADOS DO TIME'!D20:O20)</f>
         <v>0</v>
       </c>
-      <c r="G6" s="42">
+      <c r="G6" s="33">
         <f>'DADOS DO TIME'!D42+'DADOS DO TIME'!E42+'DADOS DO TIME'!F42+'DADOS DO TIME'!G42+'DADOS DO TIME'!H42+'DADOS DO TIME'!I42+'DADOS DO TIME'!J42+'DADOS DO TIME'!K42+'DADOS DO TIME'!N42+'DADOS DO TIME'!O42</f>
         <v>0</v>
       </c>
-      <c r="H6" s="66">
+      <c r="H6" s="50">
         <f>IFERROR(AVERAGE('DADOS DO TIME'!D42,'DADOS DO TIME'!E42,'DADOS DO TIME'!F42,'DADOS DO TIME'!G42,'DADOS DO TIME'!H42,'DADOS DO TIME'!I42,'DADOS DO TIME'!J42,'DADOS DO TIME'!K42,'DADOS DO TIME'!N42,'DADOS DO TIME'!O42),0)</f>
         <v>0</v>
       </c>
-      <c r="I6" s="67">
+      <c r="I6" s="51">
         <f>SUM('DADOS DO TIME'!D31:O31)</f>
         <v>0</v>
       </c>
-      <c r="J6" s="67">
+      <c r="J6" s="51">
         <f>IFERROR(AVERAGE('DADOS DO TIME'!D31,'DADOS DO TIME'!E31,'DADOS DO TIME'!F31,'DADOS DO TIME'!G31,'DADOS DO TIME'!H31,'DADOS DO TIME'!I31,'DADOS DO TIME'!J31,'DADOS DO TIME'!K31,'DADOS DO TIME'!N31,'DADOS DO TIME'!O31),0)</f>
         <v>0</v>
       </c>
-      <c r="K6" s="68">
+      <c r="K6" s="52">
         <f>COUNT('DADOS DO TIME'!D8,'DADOS DO TIME'!E8,'DADOS DO TIME'!F8,'DADOS DO TIME'!G8,'DADOS DO TIME'!H8,'DADOS DO TIME'!I8,'DADOS DO TIME'!J8,'DADOS DO TIME'!K8,'DADOS DO TIME'!N8,'DADOS DO TIME'!O8)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="2:33" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C7" s="75" t="str">
+      <c r="C7" s="59" t="str">
         <f>'DADOS DO TIME'!C9</f>
         <v>JOGADOR 3</v>
       </c>
-      <c r="D7" s="65">
+      <c r="D7" s="49">
         <f>SUM('DADOS DO TIME'!D9:O9)</f>
         <v>0</v>
       </c>
-      <c r="E7" s="66">
+      <c r="E7" s="50">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F7" s="42">
+      <c r="F7" s="33">
         <f>SUM('DADOS DO TIME'!D21:O21)</f>
         <v>0</v>
       </c>
-      <c r="G7" s="42">
+      <c r="G7" s="33">
         <f>'DADOS DO TIME'!D43+'DADOS DO TIME'!E43+'DADOS DO TIME'!F43+'DADOS DO TIME'!G43+'DADOS DO TIME'!H43+'DADOS DO TIME'!I43+'DADOS DO TIME'!J43+'DADOS DO TIME'!K43+'DADOS DO TIME'!N43+'DADOS DO TIME'!O43</f>
         <v>0</v>
       </c>
-      <c r="H7" s="66">
+      <c r="H7" s="50">
         <f>IFERROR(AVERAGE('DADOS DO TIME'!D43,'DADOS DO TIME'!E43,'DADOS DO TIME'!F43,'DADOS DO TIME'!G43,'DADOS DO TIME'!H43,'DADOS DO TIME'!I43,'DADOS DO TIME'!J43,'DADOS DO TIME'!K43,'DADOS DO TIME'!N43,'DADOS DO TIME'!O43),0)</f>
         <v>0</v>
       </c>
-      <c r="I7" s="67">
+      <c r="I7" s="51">
         <f>SUM('DADOS DO TIME'!D32:O32)</f>
         <v>0</v>
       </c>
-      <c r="J7" s="67">
+      <c r="J7" s="51">
         <f>IFERROR(AVERAGE('DADOS DO TIME'!D32,'DADOS DO TIME'!E32,'DADOS DO TIME'!F32,'DADOS DO TIME'!G32,'DADOS DO TIME'!H32,'DADOS DO TIME'!I32,'DADOS DO TIME'!J32,'DADOS DO TIME'!K32,'DADOS DO TIME'!N32,'DADOS DO TIME'!O32),0)</f>
         <v>0</v>
       </c>
-      <c r="K7" s="68">
+      <c r="K7" s="52">
         <f>COUNT('DADOS DO TIME'!D9,'DADOS DO TIME'!E9,'DADOS DO TIME'!F9,'DADOS DO TIME'!G9,'DADOS DO TIME'!H9,'DADOS DO TIME'!I9,'DADOS DO TIME'!J9,'DADOS DO TIME'!K9,'DADOS DO TIME'!N9,'DADOS DO TIME'!O9)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="2:33" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C8" s="75" t="str">
+      <c r="C8" s="59" t="str">
         <f>'DADOS DO TIME'!C10</f>
         <v>JOGADOR 4</v>
       </c>
-      <c r="D8" s="65">
+      <c r="D8" s="49">
         <f>SUM('DADOS DO TIME'!D10:O10)</f>
         <v>0</v>
       </c>
-      <c r="E8" s="66">
+      <c r="E8" s="50">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F8" s="42">
+      <c r="F8" s="33">
         <f>SUM('DADOS DO TIME'!D22:O22)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="42">
+      <c r="G8" s="33">
         <f>'DADOS DO TIME'!D44+'DADOS DO TIME'!E44+'DADOS DO TIME'!F44+'DADOS DO TIME'!G44+'DADOS DO TIME'!H44+'DADOS DO TIME'!I44+'DADOS DO TIME'!J44+'DADOS DO TIME'!K44+'DADOS DO TIME'!N44+'DADOS DO TIME'!O44</f>
         <v>0</v>
       </c>
-      <c r="H8" s="66">
+      <c r="H8" s="50">
         <f>IFERROR(AVERAGE('DADOS DO TIME'!D44,'DADOS DO TIME'!E44,'DADOS DO TIME'!F44,'DADOS DO TIME'!G44,'DADOS DO TIME'!H44,'DADOS DO TIME'!I44,'DADOS DO TIME'!J44,'DADOS DO TIME'!K44,'DADOS DO TIME'!N44,'DADOS DO TIME'!O44),0)</f>
         <v>0</v>
       </c>
-      <c r="I8" s="67">
+      <c r="I8" s="51">
         <f>SUM('DADOS DO TIME'!D33:O33)</f>
         <v>0</v>
       </c>
-      <c r="J8" s="67">
+      <c r="J8" s="51">
         <f>IFERROR(AVERAGE('DADOS DO TIME'!D33,'DADOS DO TIME'!E33,'DADOS DO TIME'!F33,'DADOS DO TIME'!G33,'DADOS DO TIME'!H33,'DADOS DO TIME'!I33,'DADOS DO TIME'!J33,'DADOS DO TIME'!K33,'DADOS DO TIME'!N33,'DADOS DO TIME'!O33),0)</f>
         <v>0</v>
       </c>
-      <c r="K8" s="68">
+      <c r="K8" s="52">
         <f>COUNT('DADOS DO TIME'!D10,'DADOS DO TIME'!E10,'DADOS DO TIME'!F10,'DADOS DO TIME'!G10,'DADOS DO TIME'!H10,'DADOS DO TIME'!I10,'DADOS DO TIME'!J10,'DADOS DO TIME'!K10,'DADOS DO TIME'!N10,'DADOS DO TIME'!O10)</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="2:33" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="75" t="str">
+      <c r="C9" s="59" t="str">
         <f>'DADOS DO TIME'!C11</f>
         <v>RESERVA 1</v>
       </c>
-      <c r="D9" s="65">
+      <c r="D9" s="49">
         <f>SUM('DADOS DO TIME'!D11:O11)</f>
         <v>0</v>
       </c>
-      <c r="E9" s="66">
+      <c r="E9" s="50">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F9" s="42">
+      <c r="F9" s="33">
         <f>SUM('DADOS DO TIME'!D23:O23)</f>
-        <v>0</v>
-      </c>
-      <c r="G9" s="42">
+        <v>22</v>
+      </c>
+      <c r="G9" s="33">
         <f>'DADOS DO TIME'!D45+'DADOS DO TIME'!E45+'DADOS DO TIME'!F45+'DADOS DO TIME'!G45+'DADOS DO TIME'!H45+'DADOS DO TIME'!I45+'DADOS DO TIME'!J45+'DADOS DO TIME'!K45+'DADOS DO TIME'!N45+'DADOS DO TIME'!O45</f>
         <v>0</v>
       </c>
-      <c r="H9" s="66">
+      <c r="H9" s="50">
         <f>IFERROR(AVERAGE('DADOS DO TIME'!D45,'DADOS DO TIME'!E45,'DADOS DO TIME'!F45,'DADOS DO TIME'!G45,'DADOS DO TIME'!H45,'DADOS DO TIME'!I45,'DADOS DO TIME'!J45,'DADOS DO TIME'!K45,'DADOS DO TIME'!N45,'DADOS DO TIME'!O45),0)</f>
         <v>0</v>
       </c>
-      <c r="I9" s="67">
+      <c r="I9" s="51">
         <f>SUM('DADOS DO TIME'!D34:O34)</f>
         <v>0</v>
       </c>
-      <c r="J9" s="67">
+      <c r="J9" s="51">
         <f>IFERROR(AVERAGE('DADOS DO TIME'!D34,'DADOS DO TIME'!E34,'DADOS DO TIME'!F34,'DADOS DO TIME'!G34,'DADOS DO TIME'!H34,'DADOS DO TIME'!I34,'DADOS DO TIME'!J34,'DADOS DO TIME'!K34,'DADOS DO TIME'!N34,'DADOS DO TIME'!O34),0)</f>
         <v>0</v>
       </c>
-      <c r="K9" s="68">
+      <c r="K9" s="52">
         <f>COUNT('DADOS DO TIME'!D11,'DADOS DO TIME'!E11,'DADOS DO TIME'!F11,'DADOS DO TIME'!G11,'DADOS DO TIME'!H11,'DADOS DO TIME'!I11,'DADOS DO TIME'!J11,'DADOS DO TIME'!K11,'DADOS DO TIME'!N11,'DADOS DO TIME'!O11)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="2:33" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C10" s="75" t="str">
+      <c r="C10" s="59">
         <f>'DADOS DO TIME'!C12</f>
-        <v>RESERVA 2</v>
-      </c>
-      <c r="D10" s="65">
+        <v>0</v>
+      </c>
+      <c r="D10" s="49">
         <f>SUM('DADOS DO TIME'!D12:O12)</f>
-        <v>0</v>
-      </c>
-      <c r="E10" s="66">
+        <v>2</v>
+      </c>
+      <c r="E10" s="50">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F10" s="42">
+        <v>2</v>
+      </c>
+      <c r="F10" s="33">
         <f>SUM('DADOS DO TIME'!D24:O24)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="42">
+      <c r="G10" s="33">
         <f>'DADOS DO TIME'!D46+'DADOS DO TIME'!E46+'DADOS DO TIME'!F46+'DADOS DO TIME'!G46+'DADOS DO TIME'!H46+'DADOS DO TIME'!I46+'DADOS DO TIME'!J46+'DADOS DO TIME'!K46+'DADOS DO TIME'!N46+'DADOS DO TIME'!O46</f>
         <v>0</v>
       </c>
-      <c r="H10" s="66">
+      <c r="H10" s="50">
         <f>IFERROR(AVERAGE('DADOS DO TIME'!D46,'DADOS DO TIME'!E46,'DADOS DO TIME'!F46,'DADOS DO TIME'!G46,'DADOS DO TIME'!H46,'DADOS DO TIME'!I46,'DADOS DO TIME'!J46,'DADOS DO TIME'!K46,'DADOS DO TIME'!N46,'DADOS DO TIME'!O46),0)</f>
         <v>0</v>
       </c>
-      <c r="I10" s="67">
+      <c r="I10" s="51">
         <f>SUM('DADOS DO TIME'!D35:O35)</f>
         <v>0</v>
       </c>
-      <c r="J10" s="67">
+      <c r="J10" s="51">
         <f>IFERROR(AVERAGE('DADOS DO TIME'!D35,'DADOS DO TIME'!E35,'DADOS DO TIME'!F35,'DADOS DO TIME'!G35,'DADOS DO TIME'!H35,'DADOS DO TIME'!I35,'DADOS DO TIME'!J35,'DADOS DO TIME'!K35,'DADOS DO TIME'!N35,'DADOS DO TIME'!O35),0)</f>
         <v>0</v>
       </c>
-      <c r="K10" s="68">
+      <c r="K10" s="52">
         <f>COUNT('DADOS DO TIME'!D12,'DADOS DO TIME'!E12,'DADOS DO TIME'!F12,'DADOS DO TIME'!G12,'DADOS DO TIME'!H12,'DADOS DO TIME'!I12,'DADOS DO TIME'!J12,'DADOS DO TIME'!K12,'DADOS DO TIME'!N12,'DADOS DO TIME'!O12)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="2:33" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C11" s="75" t="str">
+      <c r="C11" s="59" t="str">
         <f>'DADOS DO TIME'!C13</f>
         <v>RESERVA 3</v>
       </c>
-      <c r="D11" s="65">
+      <c r="D11" s="49">
         <f>SUM('DADOS DO TIME'!D13:O13)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="66">
+      <c r="E11" s="50">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F11" s="42">
+      <c r="F11" s="33">
         <f>SUM('DADOS DO TIME'!D25:O25)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="42">
+      <c r="G11" s="33">
         <f>'DADOS DO TIME'!D47+'DADOS DO TIME'!E47+'DADOS DO TIME'!F47+'DADOS DO TIME'!G47+'DADOS DO TIME'!H47+'DADOS DO TIME'!I47+'DADOS DO TIME'!J47+'DADOS DO TIME'!K47+'DADOS DO TIME'!N47+'DADOS DO TIME'!O47</f>
         <v>0</v>
       </c>
-      <c r="H11" s="66">
+      <c r="H11" s="50">
         <f>IFERROR(AVERAGE('DADOS DO TIME'!D47,'DADOS DO TIME'!E47,'DADOS DO TIME'!F47,'DADOS DO TIME'!G47,'DADOS DO TIME'!H47,'DADOS DO TIME'!I47,'DADOS DO TIME'!J47,'DADOS DO TIME'!K47,'DADOS DO TIME'!N47,'DADOS DO TIME'!O47),0)</f>
         <v>0</v>
       </c>
-      <c r="I11" s="67">
+      <c r="I11" s="51">
         <f>SUM('DADOS DO TIME'!D36:O36)</f>
         <v>0</v>
       </c>
-      <c r="J11" s="67">
+      <c r="J11" s="51">
         <f>IFERROR(AVERAGE('DADOS DO TIME'!D36,'DADOS DO TIME'!E36,'DADOS DO TIME'!F36,'DADOS DO TIME'!G36,'DADOS DO TIME'!H36,'DADOS DO TIME'!I36,'DADOS DO TIME'!J36,'DADOS DO TIME'!K36,'DADOS DO TIME'!N36,'DADOS DO TIME'!O36),0)</f>
         <v>0</v>
       </c>
-      <c r="K11" s="68">
+      <c r="K11" s="52">
         <f>COUNT('DADOS DO TIME'!D13,'DADOS DO TIME'!E13,'DADOS DO TIME'!F13,'DADOS DO TIME'!G13,'DADOS DO TIME'!H13,'DADOS DO TIME'!I13,'DADOS DO TIME'!J13,'DADOS DO TIME'!K13,'DADOS DO TIME'!N13,'DADOS DO TIME'!O13)</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="2:33" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C12" s="76" t="str">
+      <c r="C12" s="60" t="str">
         <f>'DADOS DO TIME'!C14</f>
         <v>RESERVA 4</v>
       </c>
-      <c r="D12" s="69">
+      <c r="D12" s="53">
         <f>SUM('DADOS DO TIME'!D14:O14)</f>
         <v>0</v>
       </c>
-      <c r="E12" s="70">
+      <c r="E12" s="54">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F12" s="71">
+      <c r="F12" s="55">
         <f>SUM('DADOS DO TIME'!D26:O26)</f>
         <v>0</v>
       </c>
-      <c r="G12" s="71">
+      <c r="G12" s="55">
         <f>'DADOS DO TIME'!D48+'DADOS DO TIME'!E48+'DADOS DO TIME'!F48+'DADOS DO TIME'!G48+'DADOS DO TIME'!H48+'DADOS DO TIME'!I48+'DADOS DO TIME'!J48+'DADOS DO TIME'!K48+'DADOS DO TIME'!N48+'DADOS DO TIME'!O48</f>
         <v>0</v>
       </c>
-      <c r="H12" s="70">
+      <c r="H12" s="54">
         <f>IFERROR(AVERAGE('DADOS DO TIME'!D48,'DADOS DO TIME'!E48,'DADOS DO TIME'!F48,'DADOS DO TIME'!G48,'DADOS DO TIME'!H48,'DADOS DO TIME'!I48,'DADOS DO TIME'!J48,'DADOS DO TIME'!K48,'DADOS DO TIME'!N48,'DADOS DO TIME'!O48),0)</f>
         <v>0</v>
       </c>
-      <c r="I12" s="72">
+      <c r="I12" s="56">
         <f>SUM('DADOS DO TIME'!D37:O37)</f>
         <v>0</v>
       </c>
-      <c r="J12" s="72">
+      <c r="J12" s="56">
         <f>IFERROR(AVERAGE('DADOS DO TIME'!D37,'DADOS DO TIME'!E37,'DADOS DO TIME'!F37,'DADOS DO TIME'!G37,'DADOS DO TIME'!H37,'DADOS DO TIME'!I37,'DADOS DO TIME'!J37,'DADOS DO TIME'!K37,'DADOS DO TIME'!N37,'DADOS DO TIME'!O37),0)</f>
         <v>0</v>
       </c>
-      <c r="K12" s="73">
+      <c r="K12" s="57">
         <f>COUNT('DADOS DO TIME'!D14,'DADOS DO TIME'!E14,'DADOS DO TIME'!F14,'DADOS DO TIME'!G14,'DADOS DO TIME'!H14,'DADOS DO TIME'!I14,'DADOS DO TIME'!J14,'DADOS DO TIME'!K14,'DADOS DO TIME'!N14,'DADOS DO TIME'!O14)</f>
         <v>0</v>
       </c>
@@ -6982,14 +6997,14 @@
       <c r="J16" s="13"/>
       <c r="K16" s="13"/>
       <c r="T16" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="U16" s="14">
         <f>COUNTA('DADOS DO TIME'!D5:O5)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V16" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="W16" s="14"/>
       <c r="X16" s="14"/>
@@ -6997,22 +7012,22 @@
       <c r="Z16" s="14"/>
       <c r="AA16" s="14">
         <f>SUM('DADOS DO TIME'!D7:O14)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AB16" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="AC16" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="AD16" s="14"/>
       <c r="AE16" s="14"/>
       <c r="AF16" s="14">
         <f>COUNTIF('DADOS DO TIME'!D5:O5,"&lt;4")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG16" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" spans="3:20" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -7022,29 +7037,29 @@
       <c r="K17" s="13"/>
     </row>
     <row r="18" spans="3:20" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C18" s="52" t="s">
-        <v>23</v>
-      </c>
-      <c r="D18" s="53"/>
-      <c r="E18" s="53"/>
-      <c r="F18" s="54"/>
+      <c r="C18" s="86" t="s">
+        <v>22</v>
+      </c>
+      <c r="D18" s="87"/>
+      <c r="E18" s="87"/>
+      <c r="F18" s="88"/>
       <c r="H18" s="13"/>
       <c r="I18" s="13"/>
       <c r="J18" s="13"/>
       <c r="K18" s="13"/>
     </row>
     <row r="19" spans="3:20" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C19" s="77" t="s">
+      <c r="C19" s="61" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="62" t="s">
+        <v>3</v>
+      </c>
+      <c r="E19" s="62" t="s">
         <v>24</v>
       </c>
-      <c r="D19" s="78" t="s">
-        <v>3</v>
-      </c>
-      <c r="E19" s="78" t="s">
+      <c r="F19" s="63" t="s">
         <v>25</v>
-      </c>
-      <c r="F19" s="79" t="s">
-        <v>26</v>
       </c>
       <c r="H19" s="13"/>
       <c r="I19" s="13"/>
@@ -7052,10 +7067,10 @@
       <c r="K19" s="13"/>
     </row>
     <row r="20" spans="3:20" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C20" s="80" t="s">
-        <v>31</v>
-      </c>
-      <c r="D20" s="81" t="str">
+      <c r="C20" s="64" t="s">
+        <v>30</v>
+      </c>
+      <c r="D20" s="65" t="str">
         <f>'DADOS DO TIME'!D4</f>
         <v>BERMUDA</v>
       </c>
@@ -7073,10 +7088,10 @@
       <c r="K20" s="13"/>
     </row>
     <row r="21" spans="3:20" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C21" s="80" t="s">
-        <v>32</v>
-      </c>
-      <c r="D21" s="81" t="str">
+      <c r="C21" s="64" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" s="65" t="str">
         <f>'DADOS DO TIME'!E4</f>
         <v>PURGATÓRIO</v>
       </c>
@@ -7094,10 +7109,10 @@
       <c r="K21" s="13"/>
     </row>
     <row r="22" spans="3:20" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C22" s="80" t="s">
-        <v>33</v>
-      </c>
-      <c r="D22" s="81" t="str">
+      <c r="C22" s="64" t="s">
+        <v>32</v>
+      </c>
+      <c r="D22" s="65" t="str">
         <f>'DADOS DO TIME'!F4</f>
         <v>KALAHARI</v>
       </c>
@@ -7115,10 +7130,10 @@
       <c r="K22" s="13"/>
     </row>
     <row r="23" spans="3:20" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C23" s="80" t="s">
-        <v>34</v>
-      </c>
-      <c r="D23" s="81" t="str">
+      <c r="C23" s="64" t="s">
+        <v>33</v>
+      </c>
+      <c r="D23" s="65" t="str">
         <f>'DADOS DO TIME'!G4</f>
         <v>NOVA TERRA</v>
       </c>
@@ -7136,10 +7151,10 @@
       <c r="K23" s="13"/>
     </row>
     <row r="24" spans="3:20" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C24" s="80" t="s">
-        <v>35</v>
-      </c>
-      <c r="D24" s="81" t="str">
+      <c r="C24" s="64" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" s="65" t="str">
         <f>'DADOS DO TIME'!H4</f>
         <v>ALPINE</v>
       </c>
@@ -7157,10 +7172,10 @@
       <c r="K24" s="13"/>
     </row>
     <row r="25" spans="3:20" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C25" s="80" t="s">
-        <v>36</v>
-      </c>
-      <c r="D25" s="81" t="str">
+      <c r="C25" s="64" t="s">
+        <v>35</v>
+      </c>
+      <c r="D25" s="65" t="str">
         <f>'DADOS DO TIME'!I4</f>
         <v>SOLARA</v>
       </c>
@@ -7178,14 +7193,14 @@
       <c r="K25" s="13"/>
       <c r="T25" s="1" t="str">
         <f>_xlfn.CONCAT(T16," ",U16," ",V16," ",AA16," ",AB16," ",AC16," ",AJ23," ",AF16," ",AG16)</f>
-        <v>DE 0 PARTIDAS JOGADAS O TIME ACUMULOU UM TOTAL DE 0 KILLS, E FICOU ENTRE OS 3 PRIMEIROS  0 VEZ(ES)!</v>
+        <v>DE 1 PARTIDAS JOGADAS O TIME ACUMULOU UM TOTAL DE 2 KILLS, E FICOU ENTRE OS 3 PRIMEIROS  1 VEZ(ES)!</v>
       </c>
     </row>
     <row r="26" spans="3:20" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C26" s="80" t="s">
-        <v>37</v>
-      </c>
-      <c r="D26" s="81" t="str">
+      <c r="C26" s="64" t="s">
+        <v>36</v>
+      </c>
+      <c r="D26" s="65" t="str">
         <f>'DADOS DO TIME'!J4</f>
         <v>BERMUDA</v>
       </c>
@@ -7203,10 +7218,10 @@
       <c r="K26" s="13"/>
     </row>
     <row r="27" spans="3:20" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C27" s="80" t="s">
-        <v>38</v>
-      </c>
-      <c r="D27" s="81" t="str">
+      <c r="C27" s="64" t="s">
+        <v>37</v>
+      </c>
+      <c r="D27" s="65" t="str">
         <f>'DADOS DO TIME'!K4</f>
         <v>PURGATÓRIO</v>
       </c>
@@ -7224,10 +7239,10 @@
       <c r="K27" s="17"/>
     </row>
     <row r="28" spans="3:20" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C28" s="80" t="s">
-        <v>39</v>
-      </c>
-      <c r="D28" s="81" t="str">
+      <c r="C28" s="64" t="s">
+        <v>38</v>
+      </c>
+      <c r="D28" s="65" t="str">
         <f>'DADOS DO TIME'!N4</f>
         <v>ALPINE</v>
       </c>
@@ -7241,34 +7256,34 @@
       </c>
     </row>
     <row r="29" spans="3:20" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C29" s="80" t="s">
-        <v>40</v>
-      </c>
-      <c r="D29" s="81" t="str">
+      <c r="C29" s="64" t="s">
+        <v>39</v>
+      </c>
+      <c r="D29" s="65" t="str">
         <f>'DADOS DO TIME'!O4</f>
         <v>SOLARA</v>
       </c>
       <c r="E29" s="15">
         <f>'DADOS DO TIME'!O7+'DADOS DO TIME'!O8+'DADOS DO TIME'!O9+'DADOS DO TIME'!O10+'DADOS DO TIME'!O11+'DADOS DO TIME'!O12+'DADOS DO TIME'!O13+'DADOS DO TIME'!O14</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F29" s="16">
         <f>'DADOS DO TIME'!O15</f>
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="3:20" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C30" s="82" t="s">
-        <v>11</v>
-      </c>
-      <c r="D30" s="83"/>
-      <c r="E30" s="84">
+      <c r="C30" s="91" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="92"/>
+      <c r="E30" s="66">
         <f>E20+E21+E22+E23+E24+E25+E26+E27+E28+E29</f>
-        <v>0</v>
-      </c>
-      <c r="F30" s="85">
+        <v>2</v>
+      </c>
+      <c r="F30" s="67">
         <f>'DADOS DO TIME'!D15+'DADOS DO TIME'!E15+'DADOS DO TIME'!F15+'DADOS DO TIME'!G15+'DADOS DO TIME'!H15+'DADOS DO TIME'!I15+'DADOS DO TIME'!J15+'DADOS DO TIME'!K15+'DADOS DO TIME'!N15+'DADOS DO TIME'!O15</f>
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -7336,7 +7351,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDED0EF6-6849-4010-97FD-80182192D9F9}">
-  <dimension ref="A3:X53"/>
+  <dimension ref="A3:X32"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="18" customWidth="1"/>
@@ -7356,202 +7371,202 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:24" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="33" t="s">
-        <v>30</v>
-      </c>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
+      <c r="C3" s="93" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="93"/>
+      <c r="E3" s="93"/>
+      <c r="F3" s="93"/>
+      <c r="G3" s="93"/>
     </row>
     <row r="4" spans="3:24" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="86" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="86" t="s">
+      <c r="C4" s="68" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="68" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="68" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="86" t="s">
+      <c r="F4" s="68" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="68" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="86" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="86" t="s">
-        <v>26</v>
-      </c>
     </row>
     <row r="5" spans="3:24" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="87"/>
-      <c r="D5" s="88"/>
-      <c r="E5" s="88"/>
-      <c r="F5" s="89">
+      <c r="C5" s="69"/>
+      <c r="D5" s="70"/>
+      <c r="E5" s="70"/>
+      <c r="F5" s="71">
         <f>IFERROR(E5/D5,0)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="88"/>
+      <c r="G5" s="70"/>
     </row>
     <row r="6" spans="3:24" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="87"/>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="89">
+      <c r="C6" s="69"/>
+      <c r="D6" s="70"/>
+      <c r="E6" s="70"/>
+      <c r="F6" s="71">
         <f t="shared" ref="F6:F16" si="0">IFERROR(E6/D6,0)</f>
         <v>0</v>
       </c>
-      <c r="G6" s="88"/>
+      <c r="G6" s="70"/>
     </row>
     <row r="7" spans="3:24" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C7" s="87"/>
-      <c r="D7" s="88"/>
-      <c r="E7" s="88"/>
-      <c r="F7" s="89">
+      <c r="C7" s="69"/>
+      <c r="D7" s="70"/>
+      <c r="E7" s="70"/>
+      <c r="F7" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G7" s="88"/>
+      <c r="G7" s="70"/>
     </row>
     <row r="8" spans="3:24" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C8" s="87"/>
-      <c r="D8" s="88"/>
-      <c r="E8" s="88"/>
-      <c r="F8" s="89">
+      <c r="C8" s="69"/>
+      <c r="D8" s="70"/>
+      <c r="E8" s="70"/>
+      <c r="F8" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G8" s="88"/>
+      <c r="G8" s="70"/>
     </row>
     <row r="9" spans="3:24" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="87"/>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="89">
+      <c r="C9" s="69"/>
+      <c r="D9" s="70"/>
+      <c r="E9" s="70"/>
+      <c r="F9" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G9" s="88"/>
+      <c r="G9" s="70"/>
     </row>
     <row r="10" spans="3:24" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C10" s="87"/>
-      <c r="D10" s="88"/>
-      <c r="E10" s="88"/>
-      <c r="F10" s="89">
+      <c r="C10" s="69"/>
+      <c r="D10" s="70"/>
+      <c r="E10" s="70"/>
+      <c r="F10" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G10" s="88"/>
+      <c r="G10" s="70"/>
       <c r="P10" s="19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="Q10" s="19">
         <f>COUNTA(C5:C16)</f>
         <v>0</v>
       </c>
       <c r="R10" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="S10" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="T10" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="U10" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="V10" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="W10" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="X10" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="S10" s="19" t="s">
-        <v>25</v>
-      </c>
-      <c r="T10" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="U10" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="V10" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="W10" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="X10" s="19" t="s">
-        <v>52</v>
-      </c>
     </row>
     <row r="11" spans="3:24" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C11" s="87"/>
-      <c r="D11" s="88"/>
-      <c r="E11" s="88"/>
-      <c r="F11" s="89">
+      <c r="C11" s="69"/>
+      <c r="D11" s="70"/>
+      <c r="E11" s="70"/>
+      <c r="F11" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G11" s="88"/>
+      <c r="G11" s="70"/>
     </row>
     <row r="12" spans="3:24" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C12" s="87"/>
-      <c r="D12" s="88"/>
-      <c r="E12" s="88"/>
-      <c r="F12" s="89">
+      <c r="C12" s="69"/>
+      <c r="D12" s="70"/>
+      <c r="E12" s="70"/>
+      <c r="F12" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G12" s="88"/>
+      <c r="G12" s="70"/>
     </row>
     <row r="13" spans="3:24" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C13" s="87"/>
-      <c r="D13" s="88"/>
-      <c r="E13" s="88"/>
-      <c r="F13" s="89">
+      <c r="C13" s="69"/>
+      <c r="D13" s="70"/>
+      <c r="E13" s="70"/>
+      <c r="F13" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G13" s="88"/>
+      <c r="G13" s="70"/>
     </row>
     <row r="14" spans="3:24" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C14" s="87"/>
-      <c r="D14" s="88"/>
-      <c r="E14" s="88"/>
-      <c r="F14" s="89">
+      <c r="C14" s="69"/>
+      <c r="D14" s="70"/>
+      <c r="E14" s="70"/>
+      <c r="F14" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G14" s="88"/>
+      <c r="G14" s="70"/>
       <c r="I14" s="20"/>
     </row>
     <row r="15" spans="3:24" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C15" s="87"/>
-      <c r="D15" s="88"/>
-      <c r="E15" s="88"/>
-      <c r="F15" s="89">
+      <c r="C15" s="69"/>
+      <c r="D15" s="70"/>
+      <c r="E15" s="70"/>
+      <c r="F15" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G15" s="88"/>
+      <c r="G15" s="70"/>
       <c r="Q15" s="21">
         <f>ROUND(F17,1)</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="3:24" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C16" s="87"/>
-      <c r="D16" s="88"/>
-      <c r="E16" s="88"/>
-      <c r="F16" s="89">
+      <c r="C16" s="69"/>
+      <c r="D16" s="70"/>
+      <c r="E16" s="70"/>
+      <c r="F16" s="71">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G16" s="88"/>
+      <c r="G16" s="70"/>
       <c r="Q16" s="22"/>
     </row>
     <row r="17" spans="3:20" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C17" s="86" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="90">
+      <c r="C17" s="68" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="72">
         <f>SUM(D5:D16)</f>
         <v>0</v>
       </c>
-      <c r="E17" s="90">
+      <c r="E17" s="72">
         <f>SUM(E5:E16)</f>
         <v>0</v>
       </c>
-      <c r="F17" s="91">
+      <c r="F17" s="73">
         <f>SUM(F5:F16)</f>
         <v>0</v>
       </c>
-      <c r="G17" s="90">
+      <c r="G17" s="72">
         <f>SUM(G5:G16)</f>
         <v>0</v>
       </c>
@@ -7563,11 +7578,11 @@
       <c r="N18" s="22"/>
     </row>
     <row r="19" spans="3:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P19" s="34"/>
-      <c r="Q19" s="34"/>
-      <c r="R19" s="34"/>
-      <c r="S19" s="34"/>
-      <c r="T19" s="34"/>
+      <c r="P19" s="94"/>
+      <c r="Q19" s="94"/>
+      <c r="R19" s="94"/>
+      <c r="S19" s="94"/>
+      <c r="T19" s="94"/>
     </row>
     <row r="20" spans="3:20" x14ac:dyDescent="0.25">
       <c r="Q20" s="25"/>
@@ -7600,27 +7615,6 @@
     <row r="32" spans="3:20" x14ac:dyDescent="0.25">
       <c r="I32" s="30"/>
     </row>
-    <row r="33" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="34" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="35" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="36" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="37" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="38" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="39" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="40" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="41" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="42" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="43" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="44" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="45" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="46" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="47" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="48" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="49" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="50" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="51" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="52" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="53" s="18" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="0exkp1mSx/5cgFYFFv8dgwZkalp0KyiybmLOfUPr5OFRbWPYgQHSH2oTBUCvz4v7kDSFQ/cQfDfENcL9mYIN9Q==" saltValue="mkBU4xFOQAoZy1lZ7jpX0g==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="2">

</xml_diff>